<commit_message>
v7: Remove phone number, PDF colour overhaul matching web, fix circle numbers, bigger Power Hour & Tier Ref text, taller call log rows
</commit_message>
<xml_diff>
--- a/Daily_Production_Scoreboard_v6.xlsx
+++ b/Daily_Production_Scoreboard_v6.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Daily Production Scoreboard" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'Daily Production Scoreboard'!$A$1:$G$46</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Daily Production Scoreboard'!$A$1:$G$45</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -19,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="18">
+  <fonts count="17">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -44,11 +44,6 @@
       <b val="1"/>
       <color rgb="00333333"/>
       <sz val="9"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <color rgb="00999999"/>
-      <sz val="7"/>
     </font>
     <font>
       <name val="Calibri"/>
@@ -209,7 +204,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="41">
+  <cellXfs count="40">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -221,98 +216,95 @@
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="10" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="12" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="12" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="13" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="12" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="12" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="13" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="14" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="16" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="14" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="3" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="16" fillId="3" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="14" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="13" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -680,7 +672,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G46"/>
+  <dimension ref="A1:G45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3.2" customWidth="1" min="1" max="1"/>
@@ -718,550 +710,542 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="12" customHeight="1">
-      <c r="A3" s="5" t="inlineStr">
-        <is>
-          <t>(503) 290-6958</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="2" customHeight="1">
-      <c r="A4" s="1" t="n"/>
-      <c r="B4" s="1" t="n"/>
-      <c r="C4" s="1" t="n"/>
-      <c r="D4" s="1" t="n"/>
-      <c r="E4" s="1" t="n"/>
-      <c r="F4" s="1" t="n"/>
-      <c r="G4" s="1" t="n"/>
-    </row>
-    <row r="5" ht="12" customHeight="1">
+    <row r="3" ht="2" customHeight="1">
+      <c r="A3" s="1" t="n"/>
+      <c r="B3" s="1" t="n"/>
+      <c r="C3" s="1" t="n"/>
+      <c r="D3" s="1" t="n"/>
+      <c r="E3" s="1" t="n"/>
+      <c r="F3" s="1" t="n"/>
+      <c r="G3" s="1" t="n"/>
+    </row>
+    <row r="4" ht="12" customHeight="1">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>TARGET 5  —  Real Conversations Today</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="28" customHeight="1">
       <c r="A5" s="6" t="inlineStr">
         <is>
-          <t>TARGET 5  —  Real Conversations Today</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="28" customHeight="1">
-      <c r="A6" s="7" t="inlineStr">
-        <is>
           <t>①     ②     ③     ④     ⑤</t>
         </is>
       </c>
-      <c r="D6" s="8" t="inlineStr">
+      <c r="D5" s="7" t="inlineStr">
         <is>
           <t>CALLS</t>
         </is>
       </c>
-      <c r="E6" s="8" t="inlineStr">
+      <c r="E5" s="7" t="inlineStr">
         <is>
           <t>APPTS</t>
         </is>
       </c>
-      <c r="F6" s="8" t="inlineStr">
+      <c r="F5" s="7" t="inlineStr">
         <is>
           <t>FOLLOW</t>
         </is>
       </c>
-      <c r="G6" s="8" t="inlineStr">
+      <c r="G5" s="7" t="inlineStr">
         <is>
           <t>HIT 5?</t>
         </is>
       </c>
     </row>
-    <row r="7" ht="16" customHeight="1">
-      <c r="A7" s="9" t="inlineStr">
+    <row r="6" ht="16" customHeight="1">
+      <c r="A6" s="8" t="inlineStr">
         <is>
           <t>HIT TARGET?  YES  /  NO       If not, why: _______________________________</t>
         </is>
       </c>
-      <c r="D7" s="10" t="n"/>
-      <c r="E7" s="10" t="n"/>
-      <c r="F7" s="10" t="n"/>
-      <c r="G7" s="11" t="inlineStr">
+      <c r="D6" s="9" t="n"/>
+      <c r="E6" s="9" t="n"/>
+      <c r="F6" s="9" t="n"/>
+      <c r="G6" s="10" t="inlineStr">
         <is>
           <t>Y  /  N</t>
         </is>
       </c>
     </row>
-    <row r="8" ht="2" customHeight="1">
-      <c r="A8" s="1" t="n"/>
-      <c r="B8" s="1" t="n"/>
-      <c r="C8" s="1" t="n"/>
-      <c r="D8" s="1" t="n"/>
-      <c r="E8" s="1" t="n"/>
-      <c r="F8" s="1" t="n"/>
-      <c r="G8" s="1" t="n"/>
-    </row>
-    <row r="9" ht="16" customHeight="1">
-      <c r="A9" s="12" t="inlineStr">
+    <row r="7" ht="2" customHeight="1">
+      <c r="A7" s="1" t="n"/>
+      <c r="B7" s="1" t="n"/>
+      <c r="C7" s="1" t="n"/>
+      <c r="D7" s="1" t="n"/>
+      <c r="E7" s="1" t="n"/>
+      <c r="F7" s="1" t="n"/>
+      <c r="G7" s="1" t="n"/>
+    </row>
+    <row r="8" ht="16" customHeight="1">
+      <c r="A8" s="11" t="inlineStr">
         <is>
           <t xml:space="preserve">  CALL LOG</t>
         </is>
       </c>
-      <c r="F9" s="13" t="inlineStr">
+      <c r="F8" s="12" t="inlineStr">
         <is>
           <t>S=Spoke  VM=VM  A=Appt  NA=NoAns  B=Bad#  CB=CB</t>
         </is>
       </c>
     </row>
-    <row r="10" ht="14" customHeight="1">
-      <c r="A10" s="14" t="inlineStr">
+    <row r="9" ht="14" customHeight="1">
+      <c r="A9" s="13" t="inlineStr">
         <is>
           <t>#</t>
         </is>
       </c>
-      <c r="B10" s="14" t="inlineStr">
+      <c r="B9" s="13" t="inlineStr">
         <is>
           <t>NAME</t>
         </is>
       </c>
-      <c r="C10" s="14" t="inlineStr">
+      <c r="C9" s="13" t="inlineStr">
         <is>
           <t>TIER</t>
         </is>
       </c>
-      <c r="D10" s="14" t="inlineStr">
+      <c r="D9" s="13" t="inlineStr">
         <is>
           <t>RESULT (circle)</t>
         </is>
       </c>
-      <c r="E10" s="14" t="inlineStr">
+      <c r="E9" s="13" t="inlineStr">
         <is>
           <t>NEXT STEP</t>
         </is>
       </c>
-      <c r="F10" s="15" t="n"/>
-      <c r="G10" s="15" t="n"/>
+      <c r="F9" s="14" t="n"/>
+      <c r="G9" s="14" t="n"/>
+    </row>
+    <row r="10" ht="18" customHeight="1">
+      <c r="A10" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="B10" s="16" t="n"/>
+      <c r="C10" s="17" t="inlineStr">
+        <is>
+          <t>T1  T2  T3</t>
+        </is>
+      </c>
+      <c r="D10" s="18" t="inlineStr">
+        <is>
+          <t>S  VM  A  NA  B  CB</t>
+        </is>
+      </c>
+      <c r="E10" s="16" t="n"/>
+      <c r="F10" s="19" t="n"/>
+      <c r="G10" s="19" t="n"/>
     </row>
     <row r="11" ht="18" customHeight="1">
-      <c r="A11" s="16" t="n">
-        <v>1</v>
-      </c>
-      <c r="B11" s="17" t="n"/>
-      <c r="C11" s="18" t="inlineStr">
-        <is>
-          <t>T1  T2  T3</t>
-        </is>
-      </c>
-      <c r="D11" s="19" t="inlineStr">
-        <is>
-          <t>S  VM  A  NA  B  CB</t>
-        </is>
-      </c>
-      <c r="E11" s="17" t="n"/>
-      <c r="F11" s="20" t="n"/>
-      <c r="G11" s="20" t="n"/>
+      <c r="A11" s="20" t="n">
+        <v>2</v>
+      </c>
+      <c r="B11" s="21" t="n"/>
+      <c r="C11" s="22" t="inlineStr"/>
+      <c r="D11" s="23" t="inlineStr"/>
+      <c r="E11" s="21" t="n"/>
+      <c r="F11" s="24" t="n"/>
+      <c r="G11" s="24" t="n"/>
     </row>
     <row r="12" ht="18" customHeight="1">
-      <c r="A12" s="21" t="n">
-        <v>2</v>
-      </c>
-      <c r="B12" s="22" t="n"/>
-      <c r="C12" s="23" t="inlineStr"/>
-      <c r="D12" s="24" t="inlineStr"/>
-      <c r="E12" s="22" t="n"/>
-      <c r="F12" s="25" t="n"/>
-      <c r="G12" s="25" t="n"/>
+      <c r="A12" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="B12" s="16" t="n"/>
+      <c r="C12" s="17" t="inlineStr"/>
+      <c r="D12" s="18" t="inlineStr"/>
+      <c r="E12" s="16" t="n"/>
+      <c r="F12" s="19" t="n"/>
+      <c r="G12" s="19" t="n"/>
     </row>
     <row r="13" ht="18" customHeight="1">
-      <c r="A13" s="16" t="n">
-        <v>3</v>
-      </c>
-      <c r="B13" s="17" t="n"/>
-      <c r="C13" s="18" t="inlineStr"/>
-      <c r="D13" s="19" t="inlineStr"/>
-      <c r="E13" s="17" t="n"/>
-      <c r="F13" s="20" t="n"/>
-      <c r="G13" s="20" t="n"/>
+      <c r="A13" s="20" t="n">
+        <v>4</v>
+      </c>
+      <c r="B13" s="21" t="n"/>
+      <c r="C13" s="22" t="inlineStr"/>
+      <c r="D13" s="23" t="inlineStr"/>
+      <c r="E13" s="21" t="n"/>
+      <c r="F13" s="24" t="n"/>
+      <c r="G13" s="24" t="n"/>
     </row>
     <row r="14" ht="18" customHeight="1">
-      <c r="A14" s="21" t="n">
-        <v>4</v>
-      </c>
-      <c r="B14" s="22" t="n"/>
-      <c r="C14" s="23" t="inlineStr"/>
-      <c r="D14" s="24" t="inlineStr"/>
-      <c r="E14" s="22" t="n"/>
-      <c r="F14" s="25" t="n"/>
-      <c r="G14" s="25" t="n"/>
+      <c r="A14" s="15" t="n">
+        <v>5</v>
+      </c>
+      <c r="B14" s="16" t="n"/>
+      <c r="C14" s="17" t="inlineStr"/>
+      <c r="D14" s="18" t="inlineStr"/>
+      <c r="E14" s="16" t="n"/>
+      <c r="F14" s="19" t="n"/>
+      <c r="G14" s="19" t="n"/>
     </row>
     <row r="15" ht="18" customHeight="1">
-      <c r="A15" s="16" t="n">
-        <v>5</v>
-      </c>
-      <c r="B15" s="17" t="n"/>
-      <c r="C15" s="18" t="inlineStr"/>
-      <c r="D15" s="19" t="inlineStr"/>
-      <c r="E15" s="17" t="n"/>
-      <c r="F15" s="20" t="n"/>
-      <c r="G15" s="20" t="n"/>
+      <c r="A15" s="20" t="n">
+        <v>6</v>
+      </c>
+      <c r="B15" s="21" t="n"/>
+      <c r="C15" s="22" t="inlineStr"/>
+      <c r="D15" s="23" t="inlineStr"/>
+      <c r="E15" s="21" t="n"/>
+      <c r="F15" s="24" t="n"/>
+      <c r="G15" s="24" t="n"/>
     </row>
     <row r="16" ht="18" customHeight="1">
-      <c r="A16" s="21" t="n">
-        <v>6</v>
-      </c>
-      <c r="B16" s="22" t="n"/>
-      <c r="C16" s="23" t="inlineStr"/>
-      <c r="D16" s="24" t="inlineStr"/>
-      <c r="E16" s="22" t="n"/>
-      <c r="F16" s="25" t="n"/>
-      <c r="G16" s="25" t="n"/>
+      <c r="A16" s="15" t="n">
+        <v>7</v>
+      </c>
+      <c r="B16" s="16" t="n"/>
+      <c r="C16" s="17" t="inlineStr"/>
+      <c r="D16" s="18" t="inlineStr"/>
+      <c r="E16" s="16" t="n"/>
+      <c r="F16" s="19" t="n"/>
+      <c r="G16" s="19" t="n"/>
     </row>
     <row r="17" ht="18" customHeight="1">
-      <c r="A17" s="16" t="n">
-        <v>7</v>
-      </c>
-      <c r="B17" s="17" t="n"/>
-      <c r="C17" s="18" t="inlineStr"/>
-      <c r="D17" s="19" t="inlineStr"/>
-      <c r="E17" s="17" t="n"/>
-      <c r="F17" s="20" t="n"/>
-      <c r="G17" s="20" t="n"/>
+      <c r="A17" s="20" t="n">
+        <v>8</v>
+      </c>
+      <c r="B17" s="21" t="n"/>
+      <c r="C17" s="22" t="inlineStr"/>
+      <c r="D17" s="23" t="inlineStr"/>
+      <c r="E17" s="21" t="n"/>
+      <c r="F17" s="24" t="n"/>
+      <c r="G17" s="24" t="n"/>
     </row>
     <row r="18" ht="18" customHeight="1">
-      <c r="A18" s="21" t="n">
-        <v>8</v>
-      </c>
-      <c r="B18" s="22" t="n"/>
-      <c r="C18" s="23" t="inlineStr"/>
-      <c r="D18" s="24" t="inlineStr"/>
-      <c r="E18" s="22" t="n"/>
-      <c r="F18" s="25" t="n"/>
-      <c r="G18" s="25" t="n"/>
+      <c r="A18" s="15" t="n">
+        <v>9</v>
+      </c>
+      <c r="B18" s="16" t="n"/>
+      <c r="C18" s="17" t="inlineStr"/>
+      <c r="D18" s="18" t="inlineStr"/>
+      <c r="E18" s="16" t="n"/>
+      <c r="F18" s="19" t="n"/>
+      <c r="G18" s="19" t="n"/>
     </row>
     <row r="19" ht="18" customHeight="1">
-      <c r="A19" s="16" t="n">
-        <v>9</v>
-      </c>
-      <c r="B19" s="17" t="n"/>
-      <c r="C19" s="18" t="inlineStr"/>
-      <c r="D19" s="19" t="inlineStr"/>
-      <c r="E19" s="17" t="n"/>
-      <c r="F19" s="20" t="n"/>
-      <c r="G19" s="20" t="n"/>
+      <c r="A19" s="20" t="n">
+        <v>10</v>
+      </c>
+      <c r="B19" s="21" t="n"/>
+      <c r="C19" s="22" t="inlineStr"/>
+      <c r="D19" s="23" t="inlineStr"/>
+      <c r="E19" s="21" t="n"/>
+      <c r="F19" s="24" t="n"/>
+      <c r="G19" s="24" t="n"/>
     </row>
     <row r="20" ht="18" customHeight="1">
-      <c r="A20" s="21" t="n">
-        <v>10</v>
-      </c>
-      <c r="B20" s="22" t="n"/>
-      <c r="C20" s="23" t="inlineStr"/>
-      <c r="D20" s="24" t="inlineStr"/>
-      <c r="E20" s="22" t="n"/>
-      <c r="F20" s="25" t="n"/>
-      <c r="G20" s="25" t="n"/>
+      <c r="A20" s="15" t="n">
+        <v>11</v>
+      </c>
+      <c r="B20" s="16" t="n"/>
+      <c r="C20" s="17" t="inlineStr"/>
+      <c r="D20" s="18" t="inlineStr"/>
+      <c r="E20" s="16" t="n"/>
+      <c r="F20" s="19" t="n"/>
+      <c r="G20" s="19" t="n"/>
     </row>
     <row r="21" ht="18" customHeight="1">
-      <c r="A21" s="16" t="n">
-        <v>11</v>
-      </c>
-      <c r="B21" s="17" t="n"/>
-      <c r="C21" s="18" t="inlineStr"/>
-      <c r="D21" s="19" t="inlineStr"/>
-      <c r="E21" s="17" t="n"/>
-      <c r="F21" s="20" t="n"/>
-      <c r="G21" s="20" t="n"/>
-    </row>
-    <row r="22" ht="18" customHeight="1">
-      <c r="A22" s="21" t="n">
+      <c r="A21" s="20" t="n">
         <v>12</v>
       </c>
-      <c r="B22" s="22" t="n"/>
-      <c r="C22" s="23" t="inlineStr"/>
-      <c r="D22" s="24" t="inlineStr"/>
-      <c r="E22" s="22" t="n"/>
-      <c r="F22" s="25" t="n"/>
-      <c r="G22" s="25" t="n"/>
-    </row>
-    <row r="23" ht="10" customHeight="1">
+      <c r="B21" s="21" t="n"/>
+      <c r="C21" s="22" t="inlineStr"/>
+      <c r="D21" s="23" t="inlineStr"/>
+      <c r="E21" s="21" t="n"/>
+      <c r="F21" s="24" t="n"/>
+      <c r="G21" s="24" t="n"/>
+    </row>
+    <row r="22" ht="10" customHeight="1">
+      <c r="A22" s="25" t="inlineStr">
+        <is>
+          <t>POWER HOUR: 1:30–2:30 PM  |  Block 2: 9:00–10:00 AM</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="22" customHeight="1">
       <c r="A23" s="26" t="inlineStr">
         <is>
-          <t>POWER HOUR: 1:30–2:30 PM  |  Block 2: 9:00–10:00 AM</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="22" customHeight="1">
-      <c r="A24" s="27" t="inlineStr">
-        <is>
           <t>TIER REFERENCE</t>
         </is>
       </c>
-      <c r="C24" s="28" t="inlineStr">
+      <c r="C23" s="27" t="inlineStr">
         <is>
           <t>T1</t>
         </is>
       </c>
-      <c r="D24" s="29" t="inlineStr">
+      <c r="D23" s="28" t="inlineStr">
         <is>
           <t>Hot Leads — Active buyers/sellers, referrals, warm follow-ups</t>
         </is>
       </c>
-      <c r="F24" s="30" t="inlineStr">
+      <c r="F23" s="29" t="inlineStr">
         <is>
           <t>T2</t>
         </is>
       </c>
-      <c r="G24" s="29" t="inlineStr">
+      <c r="G23" s="28" t="inlineStr">
         <is>
           <t>Easy Money — Past clients, sphere, sign calls</t>
         </is>
       </c>
     </row>
-    <row r="25" ht="14" customHeight="1">
-      <c r="A25" s="31" t="inlineStr"/>
-      <c r="C25" s="32" t="inlineStr">
+    <row r="24" ht="14" customHeight="1">
+      <c r="A24" s="30" t="inlineStr"/>
+      <c r="C24" s="31" t="inlineStr">
         <is>
           <t>T3</t>
         </is>
       </c>
-      <c r="D25" s="29" t="inlineStr">
+      <c r="D24" s="28" t="inlineStr">
         <is>
           <t>Filler Calls — Cold calls, expired/FSBO, circle prospecting</t>
         </is>
       </c>
     </row>
-    <row r="26" ht="2" customHeight="1">
-      <c r="A26" s="1" t="n"/>
-      <c r="B26" s="1" t="n"/>
-      <c r="C26" s="1" t="n"/>
-      <c r="D26" s="1" t="n"/>
-      <c r="E26" s="1" t="n"/>
-      <c r="F26" s="1" t="n"/>
-      <c r="G26" s="1" t="n"/>
-    </row>
-    <row r="27" ht="14" customHeight="1">
-      <c r="A27" s="33" t="inlineStr">
+    <row r="25" ht="2" customHeight="1">
+      <c r="A25" s="1" t="n"/>
+      <c r="B25" s="1" t="n"/>
+      <c r="C25" s="1" t="n"/>
+      <c r="D25" s="1" t="n"/>
+      <c r="E25" s="1" t="n"/>
+      <c r="F25" s="1" t="n"/>
+      <c r="G25" s="1" t="n"/>
+    </row>
+    <row r="26" ht="14" customHeight="1">
+      <c r="A26" s="32" t="inlineStr">
         <is>
           <t xml:space="preserve">  FOLLOW-UPS</t>
         </is>
       </c>
-      <c r="D27" s="33" t="inlineStr">
+      <c r="D26" s="32" t="inlineStr">
         <is>
           <t xml:space="preserve">  APPOINTMENTS SET  #___   |   OPPORTUNITIES CREATED  #___</t>
         </is>
       </c>
     </row>
-    <row r="28" ht="12" customHeight="1">
-      <c r="A28" s="14" t="inlineStr">
+    <row r="27" ht="12" customHeight="1">
+      <c r="A27" s="13" t="inlineStr">
         <is>
           <t>NAME</t>
         </is>
       </c>
-      <c r="C28" s="14" t="inlineStr">
+      <c r="C27" s="13" t="inlineStr">
         <is>
           <t>WHY / NOTES</t>
         </is>
       </c>
-      <c r="D28" s="14" t="inlineStr">
+      <c r="D27" s="13" t="inlineStr">
         <is>
           <t>NAME / OPP.</t>
         </is>
       </c>
-      <c r="F28" s="14" t="inlineStr">
+      <c r="F27" s="13" t="inlineStr">
         <is>
           <t>NOTES</t>
         </is>
       </c>
     </row>
+    <row r="28" ht="16" customHeight="1">
+      <c r="A28" s="33" t="n"/>
+      <c r="B28" s="34" t="n"/>
+      <c r="C28" s="33" t="n"/>
+      <c r="D28" s="33" t="n"/>
+      <c r="E28" s="34" t="n"/>
+      <c r="F28" s="33" t="n"/>
+      <c r="G28" s="34" t="n"/>
+    </row>
     <row r="29" ht="16" customHeight="1">
-      <c r="A29" s="34" t="n"/>
-      <c r="B29" s="35" t="n"/>
-      <c r="C29" s="34" t="n"/>
-      <c r="D29" s="34" t="n"/>
-      <c r="E29" s="35" t="n"/>
-      <c r="F29" s="34" t="n"/>
-      <c r="G29" s="35" t="n"/>
+      <c r="A29" s="35" t="n"/>
+      <c r="B29" s="34" t="n"/>
+      <c r="C29" s="35" t="n"/>
+      <c r="D29" s="35" t="n"/>
+      <c r="E29" s="34" t="n"/>
+      <c r="F29" s="35" t="n"/>
+      <c r="G29" s="34" t="n"/>
     </row>
     <row r="30" ht="16" customHeight="1">
-      <c r="A30" s="36" t="n"/>
-      <c r="B30" s="35" t="n"/>
-      <c r="C30" s="36" t="n"/>
-      <c r="D30" s="36" t="n"/>
-      <c r="E30" s="35" t="n"/>
-      <c r="F30" s="36" t="n"/>
-      <c r="G30" s="35" t="n"/>
+      <c r="A30" s="33" t="n"/>
+      <c r="B30" s="34" t="n"/>
+      <c r="C30" s="33" t="n"/>
+      <c r="D30" s="33" t="n"/>
+      <c r="E30" s="34" t="n"/>
+      <c r="F30" s="33" t="n"/>
+      <c r="G30" s="34" t="n"/>
     </row>
     <row r="31" ht="16" customHeight="1">
-      <c r="A31" s="34" t="n"/>
-      <c r="B31" s="35" t="n"/>
-      <c r="C31" s="34" t="n"/>
-      <c r="D31" s="34" t="n"/>
-      <c r="E31" s="35" t="n"/>
-      <c r="F31" s="34" t="n"/>
-      <c r="G31" s="35" t="n"/>
+      <c r="A31" s="35" t="n"/>
+      <c r="B31" s="34" t="n"/>
+      <c r="C31" s="35" t="n"/>
+      <c r="D31" s="35" t="n"/>
+      <c r="E31" s="34" t="n"/>
+      <c r="F31" s="35" t="n"/>
+      <c r="G31" s="34" t="n"/>
     </row>
     <row r="32" ht="16" customHeight="1">
-      <c r="A32" s="36" t="n"/>
-      <c r="B32" s="35" t="n"/>
-      <c r="C32" s="36" t="n"/>
-      <c r="D32" s="36" t="n"/>
-      <c r="E32" s="35" t="n"/>
-      <c r="F32" s="36" t="n"/>
-      <c r="G32" s="35" t="n"/>
-    </row>
-    <row r="33" ht="16" customHeight="1">
-      <c r="A33" s="34" t="n"/>
-      <c r="B33" s="35" t="n"/>
-      <c r="C33" s="34" t="n"/>
-      <c r="D33" s="34" t="n"/>
-      <c r="E33" s="35" t="n"/>
-      <c r="F33" s="34" t="n"/>
-      <c r="G33" s="35" t="n"/>
-    </row>
-    <row r="34" ht="2" customHeight="1">
-      <c r="A34" s="1" t="n"/>
-      <c r="B34" s="1" t="n"/>
-      <c r="C34" s="1" t="n"/>
-      <c r="D34" s="1" t="n"/>
-      <c r="E34" s="1" t="n"/>
-      <c r="F34" s="1" t="n"/>
-      <c r="G34" s="1" t="n"/>
-    </row>
-    <row r="35" ht="16" customHeight="1">
-      <c r="A35" s="12" t="inlineStr">
+      <c r="A32" s="33" t="n"/>
+      <c r="B32" s="34" t="n"/>
+      <c r="C32" s="33" t="n"/>
+      <c r="D32" s="33" t="n"/>
+      <c r="E32" s="34" t="n"/>
+      <c r="F32" s="33" t="n"/>
+      <c r="G32" s="34" t="n"/>
+    </row>
+    <row r="33" ht="2" customHeight="1">
+      <c r="A33" s="1" t="n"/>
+      <c r="B33" s="1" t="n"/>
+      <c r="C33" s="1" t="n"/>
+      <c r="D33" s="1" t="n"/>
+      <c r="E33" s="1" t="n"/>
+      <c r="F33" s="1" t="n"/>
+      <c r="G33" s="1" t="n"/>
+    </row>
+    <row r="34" ht="16" customHeight="1">
+      <c r="A34" s="11" t="inlineStr">
         <is>
           <t xml:space="preserve">  DAILY REVIEW</t>
         </is>
       </c>
     </row>
-    <row r="36" ht="12" customHeight="1">
-      <c r="A36" s="37" t="inlineStr">
+    <row r="35" ht="12" customHeight="1">
+      <c r="A35" s="36" t="inlineStr">
         <is>
           <t xml:space="preserve">  WHAT DIDN'T WORK?</t>
         </is>
       </c>
     </row>
+    <row r="36" ht="16" customHeight="1">
+      <c r="A36" s="37" t="inlineStr"/>
+      <c r="B36" s="38" t="n"/>
+      <c r="C36" s="38" t="n"/>
+      <c r="D36" s="38" t="n"/>
+      <c r="E36" s="38" t="n"/>
+      <c r="F36" s="38" t="n"/>
+      <c r="G36" s="38" t="n"/>
+    </row>
     <row r="37" ht="16" customHeight="1">
-      <c r="A37" s="38" t="inlineStr"/>
-      <c r="B37" s="39" t="n"/>
-      <c r="C37" s="39" t="n"/>
-      <c r="D37" s="39" t="n"/>
-      <c r="E37" s="39" t="n"/>
-      <c r="F37" s="39" t="n"/>
-      <c r="G37" s="39" t="n"/>
-    </row>
-    <row r="38" ht="16" customHeight="1">
-      <c r="A38" s="38" t="inlineStr"/>
-      <c r="B38" s="39" t="n"/>
-      <c r="C38" s="39" t="n"/>
-      <c r="D38" s="39" t="n"/>
-      <c r="E38" s="39" t="n"/>
-      <c r="F38" s="39" t="n"/>
-      <c r="G38" s="39" t="n"/>
-    </row>
-    <row r="39" ht="12" customHeight="1">
-      <c r="A39" s="37" t="inlineStr">
+      <c r="A37" s="37" t="inlineStr"/>
+      <c r="B37" s="38" t="n"/>
+      <c r="C37" s="38" t="n"/>
+      <c r="D37" s="38" t="n"/>
+      <c r="E37" s="38" t="n"/>
+      <c r="F37" s="38" t="n"/>
+      <c r="G37" s="38" t="n"/>
+    </row>
+    <row r="38" ht="12" customHeight="1">
+      <c r="A38" s="36" t="inlineStr">
         <is>
           <t xml:space="preserve">  WHAT WORKED TODAY?</t>
         </is>
       </c>
     </row>
+    <row r="39" ht="16" customHeight="1">
+      <c r="A39" s="37" t="inlineStr"/>
+      <c r="B39" s="38" t="n"/>
+      <c r="C39" s="38" t="n"/>
+      <c r="D39" s="38" t="n"/>
+      <c r="E39" s="38" t="n"/>
+      <c r="F39" s="38" t="n"/>
+      <c r="G39" s="38" t="n"/>
+    </row>
     <row r="40" ht="16" customHeight="1">
-      <c r="A40" s="38" t="inlineStr"/>
-      <c r="B40" s="39" t="n"/>
-      <c r="C40" s="39" t="n"/>
-      <c r="D40" s="39" t="n"/>
-      <c r="E40" s="39" t="n"/>
-      <c r="F40" s="39" t="n"/>
-      <c r="G40" s="39" t="n"/>
-    </row>
-    <row r="41" ht="16" customHeight="1">
-      <c r="A41" s="38" t="inlineStr"/>
-      <c r="B41" s="39" t="n"/>
-      <c r="C41" s="39" t="n"/>
-      <c r="D41" s="39" t="n"/>
-      <c r="E41" s="39" t="n"/>
-      <c r="F41" s="39" t="n"/>
-      <c r="G41" s="39" t="n"/>
-    </row>
-    <row r="42" ht="12" customHeight="1">
-      <c r="A42" s="37" t="inlineStr">
+      <c r="A40" s="37" t="inlineStr"/>
+      <c r="B40" s="38" t="n"/>
+      <c r="C40" s="38" t="n"/>
+      <c r="D40" s="38" t="n"/>
+      <c r="E40" s="38" t="n"/>
+      <c r="F40" s="38" t="n"/>
+      <c r="G40" s="38" t="n"/>
+    </row>
+    <row r="41" ht="12" customHeight="1">
+      <c r="A41" s="36" t="inlineStr">
         <is>
           <t xml:space="preserve">  WHAT WILL I IMPROVE TOMORROW?</t>
         </is>
       </c>
     </row>
+    <row r="42" ht="16" customHeight="1">
+      <c r="A42" s="37" t="inlineStr"/>
+      <c r="B42" s="38" t="n"/>
+      <c r="C42" s="38" t="n"/>
+      <c r="D42" s="38" t="n"/>
+      <c r="E42" s="38" t="n"/>
+      <c r="F42" s="38" t="n"/>
+      <c r="G42" s="38" t="n"/>
+    </row>
     <row r="43" ht="16" customHeight="1">
-      <c r="A43" s="38" t="inlineStr"/>
-      <c r="B43" s="39" t="n"/>
-      <c r="C43" s="39" t="n"/>
-      <c r="D43" s="39" t="n"/>
-      <c r="E43" s="39" t="n"/>
-      <c r="F43" s="39" t="n"/>
-      <c r="G43" s="39" t="n"/>
-    </row>
-    <row r="44" ht="16" customHeight="1">
-      <c r="A44" s="38" t="inlineStr"/>
-      <c r="B44" s="39" t="n"/>
-      <c r="C44" s="39" t="n"/>
-      <c r="D44" s="39" t="n"/>
-      <c r="E44" s="39" t="n"/>
-      <c r="F44" s="39" t="n"/>
-      <c r="G44" s="39" t="n"/>
-    </row>
-    <row r="45" ht="2" customHeight="1">
-      <c r="A45" s="1" t="n"/>
-      <c r="B45" s="1" t="n"/>
-      <c r="C45" s="1" t="n"/>
-      <c r="D45" s="1" t="n"/>
-      <c r="E45" s="1" t="n"/>
-      <c r="F45" s="1" t="n"/>
-      <c r="G45" s="1" t="n"/>
-    </row>
-    <row r="46" ht="12" customHeight="1">
-      <c r="A46" s="40" t="inlineStr">
+      <c r="A43" s="37" t="inlineStr"/>
+      <c r="B43" s="38" t="n"/>
+      <c r="C43" s="38" t="n"/>
+      <c r="D43" s="38" t="n"/>
+      <c r="E43" s="38" t="n"/>
+      <c r="F43" s="38" t="n"/>
+      <c r="G43" s="38" t="n"/>
+    </row>
+    <row r="44" ht="2" customHeight="1">
+      <c r="A44" s="1" t="n"/>
+      <c r="B44" s="1" t="n"/>
+      <c r="C44" s="1" t="n"/>
+      <c r="D44" s="1" t="n"/>
+      <c r="E44" s="1" t="n"/>
+      <c r="F44" s="1" t="n"/>
+      <c r="G44" s="1" t="n"/>
+    </row>
+    <row r="45" ht="12" customHeight="1">
+      <c r="A45" s="39" t="inlineStr">
         <is>
           <t>Daily Production Scoreboard  |  © 2026</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="45">
+  <mergeCells count="44">
     <mergeCell ref="A24:B24"/>
     <mergeCell ref="A30:B30"/>
     <mergeCell ref="F29:G29"/>
-    <mergeCell ref="D25:G25"/>
+    <mergeCell ref="A22:G22"/>
     <mergeCell ref="A35:G35"/>
-    <mergeCell ref="A27:C27"/>
+    <mergeCell ref="A4:G4"/>
+    <mergeCell ref="D24:G24"/>
     <mergeCell ref="A38:G38"/>
-    <mergeCell ref="A42:G42"/>
     <mergeCell ref="A43:G43"/>
     <mergeCell ref="D31:E31"/>
+    <mergeCell ref="A26:C26"/>
     <mergeCell ref="A2:C2"/>
-    <mergeCell ref="A44:G44"/>
+    <mergeCell ref="D26:G26"/>
     <mergeCell ref="F30:G30"/>
+    <mergeCell ref="D2:E2"/>
+    <mergeCell ref="A5:C5"/>
     <mergeCell ref="A40:G40"/>
-    <mergeCell ref="D2:E2"/>
-    <mergeCell ref="A25:B25"/>
     <mergeCell ref="A39:G39"/>
-    <mergeCell ref="F33:G33"/>
+    <mergeCell ref="D27:E27"/>
+    <mergeCell ref="A34:G34"/>
     <mergeCell ref="D32:E32"/>
     <mergeCell ref="F32:G32"/>
+    <mergeCell ref="A27:B27"/>
+    <mergeCell ref="A45:G45"/>
+    <mergeCell ref="F8:G8"/>
     <mergeCell ref="A36:G36"/>
     <mergeCell ref="F2:G2"/>
-    <mergeCell ref="A33:B33"/>
     <mergeCell ref="F31:G31"/>
     <mergeCell ref="D28:E28"/>
     <mergeCell ref="A32:B32"/>
     <mergeCell ref="F28:G28"/>
-    <mergeCell ref="D27:G27"/>
+    <mergeCell ref="A23:B23"/>
+    <mergeCell ref="A8:E8"/>
     <mergeCell ref="A41:G41"/>
-    <mergeCell ref="F9:G9"/>
+    <mergeCell ref="F27:G27"/>
     <mergeCell ref="A37:G37"/>
-    <mergeCell ref="A46:G46"/>
-    <mergeCell ref="D24:E24"/>
     <mergeCell ref="A29:B29"/>
     <mergeCell ref="D30:E30"/>
-    <mergeCell ref="A3:G3"/>
-    <mergeCell ref="D33:E33"/>
     <mergeCell ref="D29:E29"/>
     <mergeCell ref="A6:C6"/>
+    <mergeCell ref="D23:E23"/>
     <mergeCell ref="A28:B28"/>
-    <mergeCell ref="A7:C7"/>
     <mergeCell ref="A31:B31"/>
-    <mergeCell ref="A9:E9"/>
-    <mergeCell ref="A5:G5"/>
-    <mergeCell ref="A23:G23"/>
+    <mergeCell ref="A42:G42"/>
   </mergeCells>
   <pageMargins left="0.3" right="0.3" top="0.25" bottom="0.25" header="0.05" footer="0.05"/>
   <pageSetup orientation="portrait" paperSize="1" fitToHeight="1" fitToWidth="1"/>

</xml_diff>

<commit_message>
Update text in PDF and Excel.
</commit_message>
<xml_diff>
--- a/Daily_Production_Scoreboard_v6.xlsx
+++ b/Daily_Production_Scoreboard_v6.xlsx
@@ -978,7 +978,7 @@
       </c>
       <c r="D23" s="28" t="inlineStr">
         <is>
-          <t>Hot Leads — Active buyers/sellers, referrals, warm follow-ups</t>
+          <t>Convert fast - highest priority — Active buyers/sellers, referrals, warm follow-ups</t>
         </is>
       </c>
       <c r="F23" s="29" t="inlineStr">
@@ -988,7 +988,7 @@
       </c>
       <c r="G23" s="28" t="inlineStr">
         <is>
-          <t>Easy Money — Past clients, sphere, sign calls</t>
+          <t>Quick wins, low-hanging fruit — Past clients, sphere, sign calls</t>
         </is>
       </c>
     </row>
@@ -1001,7 +1001,7 @@
       </c>
       <c r="D24" s="28" t="inlineStr">
         <is>
-          <t>Filler Calls — Cold calls, expired/FSBO, circle prospecting</t>
+          <t>Volume calls, keep pipeline full — Cold calls, expired/FSBO, circle prospecting</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Split call log into Block 1 (Power Hour T1+T2) and Block 2 (Cleanup) across PDF, Excel, and Web
</commit_message>
<xml_diff>
--- a/Daily_Production_Scoreboard_v6.xlsx
+++ b/Daily_Production_Scoreboard_v6.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Daily Production Scoreboard" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'Daily Production Scoreboard'!$A$1:$G$45</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Daily Production Scoreboard'!$A$1:$G$48</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -19,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="17">
+  <fonts count="20">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -88,6 +88,18 @@
     </font>
     <font>
       <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="004A5568"/>
+      <sz val="7"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <i val="1"/>
+      <color rgb="00667788"/>
+      <sz val="5.5"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
       <color rgb="00CCCCCC"/>
       <sz val="7"/>
     </font>
@@ -100,6 +112,12 @@
       <name val="Calibri"/>
       <color rgb="00CCCCCC"/>
       <sz val="6"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="004A5568"/>
+      <sz val="6.5"/>
     </font>
     <font>
       <name val="Calibri"/>
@@ -118,7 +136,7 @@
       <sz val="8"/>
     </font>
   </fonts>
-  <fills count="9">
+  <fills count="13">
     <fill>
       <patternFill/>
     </fill>
@@ -141,6 +159,30 @@
       <patternFill patternType="solid">
         <fgColor rgb="00F0F0F0"/>
         <bgColor rgb="00F0F0F0"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F5F0E0"/>
+        <bgColor rgb="00F5F0E0"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E8EDF3"/>
+        <bgColor rgb="00E8EDF3"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EFF2E8"/>
+        <bgColor rgb="00EFF2E8"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00ECEEF2"/>
+        <bgColor rgb="00ECEEF2"/>
       </patternFill>
     </fill>
     <fill>
@@ -204,7 +246,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="40">
+  <cellXfs count="43">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -240,58 +282,67 @@
     <xf numFmtId="0" fontId="10" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="11" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="8" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="11" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="13" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="14" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="13" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="14" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="12" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="9" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="9" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="9" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="12" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -300,11 +351,11 @@
     <xf numFmtId="0" fontId="8" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="3" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="19" fillId="3" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="13" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="15" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -672,7 +723,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G45"/>
+  <dimension ref="A1:G48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3.2" customWidth="1" min="1" max="1"/>
@@ -792,460 +843,572 @@
     <row r="9" ht="14" customHeight="1">
       <c r="A9" s="13" t="inlineStr">
         <is>
+          <t>⏰  BLOCK 1 — The Power Hour: 1:30 – 2:30 PM</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="11" customHeight="1">
+      <c r="A10" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Tier 1 (First 30 min) — Convert fast: active leads, buyers/sellers, referrals</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="14" customHeight="1">
+      <c r="A11" s="15" t="inlineStr">
+        <is>
           <t>#</t>
         </is>
       </c>
-      <c r="B9" s="13" t="inlineStr">
+      <c r="B11" s="15" t="inlineStr">
         <is>
           <t>NAME</t>
         </is>
       </c>
-      <c r="C9" s="13" t="inlineStr">
+      <c r="C11" s="15" t="inlineStr">
         <is>
           <t>TIER</t>
         </is>
       </c>
-      <c r="D9" s="13" t="inlineStr">
+      <c r="D11" s="15" t="inlineStr">
         <is>
           <t>RESULT (circle)</t>
         </is>
       </c>
-      <c r="E9" s="13" t="inlineStr">
+      <c r="E11" s="15" t="inlineStr">
         <is>
           <t>NEXT STEP</t>
         </is>
       </c>
-      <c r="F9" s="14" t="n"/>
-      <c r="G9" s="14" t="n"/>
-    </row>
-    <row r="10" ht="18" customHeight="1">
-      <c r="A10" s="15" t="n">
+      <c r="F11" s="16" t="n"/>
+      <c r="G11" s="16" t="n"/>
+    </row>
+    <row r="12" ht="18" customHeight="1">
+      <c r="A12" s="17" t="n">
         <v>1</v>
       </c>
-      <c r="B10" s="16" t="n"/>
-      <c r="C10" s="17" t="inlineStr">
+      <c r="B12" s="18" t="n"/>
+      <c r="C12" s="19" t="inlineStr">
         <is>
           <t>T1  T2  T3</t>
         </is>
       </c>
-      <c r="D10" s="18" t="inlineStr">
+      <c r="D12" s="20" t="inlineStr">
         <is>
           <t>S  VM  A  NA  B  CB</t>
         </is>
       </c>
-      <c r="E10" s="16" t="n"/>
-      <c r="F10" s="19" t="n"/>
-      <c r="G10" s="19" t="n"/>
-    </row>
-    <row r="11" ht="18" customHeight="1">
-      <c r="A11" s="20" t="n">
+      <c r="E12" s="18" t="n"/>
+      <c r="F12" s="21" t="n"/>
+      <c r="G12" s="21" t="n"/>
+    </row>
+    <row r="13" ht="18" customHeight="1">
+      <c r="A13" s="22" t="n">
         <v>2</v>
       </c>
-      <c r="B11" s="21" t="n"/>
-      <c r="C11" s="22" t="inlineStr"/>
-      <c r="D11" s="23" t="inlineStr"/>
-      <c r="E11" s="21" t="n"/>
-      <c r="F11" s="24" t="n"/>
-      <c r="G11" s="24" t="n"/>
-    </row>
-    <row r="12" ht="18" customHeight="1">
-      <c r="A12" s="15" t="n">
+      <c r="B13" s="23" t="n"/>
+      <c r="C13" s="24" t="inlineStr">
+        <is>
+          <t>T1  T2  T3</t>
+        </is>
+      </c>
+      <c r="D13" s="25" t="inlineStr">
+        <is>
+          <t>S  VM  A  NA  B  CB</t>
+        </is>
+      </c>
+      <c r="E13" s="23" t="n"/>
+      <c r="F13" s="26" t="n"/>
+      <c r="G13" s="26" t="n"/>
+    </row>
+    <row r="14" ht="18" customHeight="1">
+      <c r="A14" s="17" t="n">
         <v>3</v>
       </c>
-      <c r="B12" s="16" t="n"/>
-      <c r="C12" s="17" t="inlineStr"/>
-      <c r="D12" s="18" t="inlineStr"/>
-      <c r="E12" s="16" t="n"/>
-      <c r="F12" s="19" t="n"/>
-      <c r="G12" s="19" t="n"/>
-    </row>
-    <row r="13" ht="18" customHeight="1">
-      <c r="A13" s="20" t="n">
+      <c r="B14" s="18" t="n"/>
+      <c r="C14" s="19" t="inlineStr">
+        <is>
+          <t>T1  T2  T3</t>
+        </is>
+      </c>
+      <c r="D14" s="20" t="inlineStr">
+        <is>
+          <t>S  VM  A  NA  B  CB</t>
+        </is>
+      </c>
+      <c r="E14" s="18" t="n"/>
+      <c r="F14" s="21" t="n"/>
+      <c r="G14" s="21" t="n"/>
+    </row>
+    <row r="15" ht="18" customHeight="1">
+      <c r="A15" s="22" t="n">
         <v>4</v>
       </c>
-      <c r="B13" s="21" t="n"/>
-      <c r="C13" s="22" t="inlineStr"/>
-      <c r="D13" s="23" t="inlineStr"/>
-      <c r="E13" s="21" t="n"/>
-      <c r="F13" s="24" t="n"/>
-      <c r="G13" s="24" t="n"/>
-    </row>
-    <row r="14" ht="18" customHeight="1">
-      <c r="A14" s="15" t="n">
+      <c r="B15" s="23" t="n"/>
+      <c r="C15" s="24" t="inlineStr">
+        <is>
+          <t>T1  T2  T3</t>
+        </is>
+      </c>
+      <c r="D15" s="25" t="inlineStr">
+        <is>
+          <t>S  VM  A  NA  B  CB</t>
+        </is>
+      </c>
+      <c r="E15" s="23" t="n"/>
+      <c r="F15" s="26" t="n"/>
+      <c r="G15" s="26" t="n"/>
+    </row>
+    <row r="16" ht="11" customHeight="1">
+      <c r="A16" s="27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Tier 2 (Second 30 min) — Quick wins: past clients, sphere, sign calls</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="18" customHeight="1">
+      <c r="A17" s="17" t="n">
         <v>5</v>
       </c>
-      <c r="B14" s="16" t="n"/>
-      <c r="C14" s="17" t="inlineStr"/>
-      <c r="D14" s="18" t="inlineStr"/>
-      <c r="E14" s="16" t="n"/>
-      <c r="F14" s="19" t="n"/>
-      <c r="G14" s="19" t="n"/>
-    </row>
-    <row r="15" ht="18" customHeight="1">
-      <c r="A15" s="20" t="n">
+      <c r="B17" s="18" t="n"/>
+      <c r="C17" s="19" t="inlineStr">
+        <is>
+          <t>T1  T2  T3</t>
+        </is>
+      </c>
+      <c r="D17" s="20" t="inlineStr">
+        <is>
+          <t>S  VM  A  NA  B  CB</t>
+        </is>
+      </c>
+      <c r="E17" s="18" t="n"/>
+      <c r="F17" s="21" t="n"/>
+      <c r="G17" s="21" t="n"/>
+    </row>
+    <row r="18" ht="18" customHeight="1">
+      <c r="A18" s="22" t="n">
         <v>6</v>
       </c>
-      <c r="B15" s="21" t="n"/>
-      <c r="C15" s="22" t="inlineStr"/>
-      <c r="D15" s="23" t="inlineStr"/>
-      <c r="E15" s="21" t="n"/>
-      <c r="F15" s="24" t="n"/>
-      <c r="G15" s="24" t="n"/>
-    </row>
-    <row r="16" ht="18" customHeight="1">
-      <c r="A16" s="15" t="n">
+      <c r="B18" s="23" t="n"/>
+      <c r="C18" s="24" t="inlineStr">
+        <is>
+          <t>T1  T2  T3</t>
+        </is>
+      </c>
+      <c r="D18" s="25" t="inlineStr">
+        <is>
+          <t>S  VM  A  NA  B  CB</t>
+        </is>
+      </c>
+      <c r="E18" s="23" t="n"/>
+      <c r="F18" s="26" t="n"/>
+      <c r="G18" s="26" t="n"/>
+    </row>
+    <row r="19" ht="18" customHeight="1">
+      <c r="A19" s="17" t="n">
         <v>7</v>
       </c>
-      <c r="B16" s="16" t="n"/>
-      <c r="C16" s="17" t="inlineStr"/>
-      <c r="D16" s="18" t="inlineStr"/>
-      <c r="E16" s="16" t="n"/>
-      <c r="F16" s="19" t="n"/>
-      <c r="G16" s="19" t="n"/>
-    </row>
-    <row r="17" ht="18" customHeight="1">
-      <c r="A17" s="20" t="n">
+      <c r="B19" s="18" t="n"/>
+      <c r="C19" s="19" t="inlineStr">
+        <is>
+          <t>T1  T2  T3</t>
+        </is>
+      </c>
+      <c r="D19" s="20" t="inlineStr">
+        <is>
+          <t>S  VM  A  NA  B  CB</t>
+        </is>
+      </c>
+      <c r="E19" s="18" t="n"/>
+      <c r="F19" s="21" t="n"/>
+      <c r="G19" s="21" t="n"/>
+    </row>
+    <row r="20" ht="18" customHeight="1">
+      <c r="A20" s="22" t="n">
         <v>8</v>
       </c>
-      <c r="B17" s="21" t="n"/>
-      <c r="C17" s="22" t="inlineStr"/>
-      <c r="D17" s="23" t="inlineStr"/>
-      <c r="E17" s="21" t="n"/>
-      <c r="F17" s="24" t="n"/>
-      <c r="G17" s="24" t="n"/>
-    </row>
-    <row r="18" ht="18" customHeight="1">
-      <c r="A18" s="15" t="n">
+      <c r="B20" s="23" t="n"/>
+      <c r="C20" s="24" t="inlineStr">
+        <is>
+          <t>T1  T2  T3</t>
+        </is>
+      </c>
+      <c r="D20" s="25" t="inlineStr">
+        <is>
+          <t>S  VM  A  NA  B  CB</t>
+        </is>
+      </c>
+      <c r="E20" s="23" t="n"/>
+      <c r="F20" s="26" t="n"/>
+      <c r="G20" s="26" t="n"/>
+    </row>
+    <row r="21" ht="14" customHeight="1">
+      <c r="A21" s="28" t="inlineStr">
+        <is>
+          <t>⏰  BLOCK 2 — The Cleanup: 4:30 – 5:00 PM  •  Circling back on earlier calls &amp; callbacks</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="18" customHeight="1">
+      <c r="A22" s="17" t="n">
         <v>9</v>
       </c>
-      <c r="B18" s="16" t="n"/>
-      <c r="C18" s="17" t="inlineStr"/>
-      <c r="D18" s="18" t="inlineStr"/>
-      <c r="E18" s="16" t="n"/>
-      <c r="F18" s="19" t="n"/>
-      <c r="G18" s="19" t="n"/>
-    </row>
-    <row r="19" ht="18" customHeight="1">
-      <c r="A19" s="20" t="n">
+      <c r="B22" s="18" t="n"/>
+      <c r="C22" s="19" t="inlineStr">
+        <is>
+          <t>T1  T2  T3</t>
+        </is>
+      </c>
+      <c r="D22" s="20" t="inlineStr">
+        <is>
+          <t>S  VM  A  NA  B  CB</t>
+        </is>
+      </c>
+      <c r="E22" s="18" t="n"/>
+      <c r="F22" s="21" t="n"/>
+      <c r="G22" s="21" t="n"/>
+    </row>
+    <row r="23" ht="18" customHeight="1">
+      <c r="A23" s="22" t="n">
         <v>10</v>
       </c>
-      <c r="B19" s="21" t="n"/>
-      <c r="C19" s="22" t="inlineStr"/>
-      <c r="D19" s="23" t="inlineStr"/>
-      <c r="E19" s="21" t="n"/>
-      <c r="F19" s="24" t="n"/>
-      <c r="G19" s="24" t="n"/>
-    </row>
-    <row r="20" ht="18" customHeight="1">
-      <c r="A20" s="15" t="n">
+      <c r="B23" s="23" t="n"/>
+      <c r="C23" s="24" t="inlineStr">
+        <is>
+          <t>T1  T2  T3</t>
+        </is>
+      </c>
+      <c r="D23" s="25" t="inlineStr">
+        <is>
+          <t>S  VM  A  NA  B  CB</t>
+        </is>
+      </c>
+      <c r="E23" s="23" t="n"/>
+      <c r="F23" s="26" t="n"/>
+      <c r="G23" s="26" t="n"/>
+    </row>
+    <row r="24" ht="18" customHeight="1">
+      <c r="A24" s="17" t="n">
         <v>11</v>
       </c>
-      <c r="B20" s="16" t="n"/>
-      <c r="C20" s="17" t="inlineStr"/>
-      <c r="D20" s="18" t="inlineStr"/>
-      <c r="E20" s="16" t="n"/>
-      <c r="F20" s="19" t="n"/>
-      <c r="G20" s="19" t="n"/>
-    </row>
-    <row r="21" ht="18" customHeight="1">
-      <c r="A21" s="20" t="n">
+      <c r="B24" s="18" t="n"/>
+      <c r="C24" s="19" t="inlineStr">
+        <is>
+          <t>T1  T2  T3</t>
+        </is>
+      </c>
+      <c r="D24" s="20" t="inlineStr">
+        <is>
+          <t>S  VM  A  NA  B  CB</t>
+        </is>
+      </c>
+      <c r="E24" s="18" t="n"/>
+      <c r="F24" s="21" t="n"/>
+      <c r="G24" s="21" t="n"/>
+    </row>
+    <row r="25" ht="18" customHeight="1">
+      <c r="A25" s="22" t="n">
         <v>12</v>
       </c>
-      <c r="B21" s="21" t="n"/>
-      <c r="C21" s="22" t="inlineStr"/>
-      <c r="D21" s="23" t="inlineStr"/>
-      <c r="E21" s="21" t="n"/>
-      <c r="F21" s="24" t="n"/>
-      <c r="G21" s="24" t="n"/>
-    </row>
-    <row r="22" ht="10" customHeight="1">
-      <c r="A22" s="25" t="inlineStr">
-        <is>
-          <t>Block 1: 1:30–2:30 PM  |  Block 2: 4:30–5:00 PM</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="22" customHeight="1">
-      <c r="A23" s="26" t="inlineStr">
+      <c r="B25" s="23" t="n"/>
+      <c r="C25" s="24" t="inlineStr">
+        <is>
+          <t>T1  T2  T3</t>
+        </is>
+      </c>
+      <c r="D25" s="25" t="inlineStr">
+        <is>
+          <t>S  VM  A  NA  B  CB</t>
+        </is>
+      </c>
+      <c r="E25" s="23" t="n"/>
+      <c r="F25" s="26" t="n"/>
+      <c r="G25" s="26" t="n"/>
+    </row>
+    <row r="26" ht="22" customHeight="1">
+      <c r="A26" s="29" t="inlineStr">
         <is>
           <t>TIER REFERENCE</t>
         </is>
       </c>
-      <c r="C23" s="27" t="inlineStr">
+      <c r="C26" s="30" t="inlineStr">
         <is>
           <t>T1</t>
         </is>
       </c>
-      <c r="D23" s="28" t="inlineStr">
+      <c r="D26" s="31" t="inlineStr">
         <is>
           <t>Convert fast - highest priority — Active buyers/sellers, referrals, warm follow-ups</t>
         </is>
       </c>
-      <c r="F23" s="29" t="inlineStr">
+      <c r="F26" s="32" t="inlineStr">
         <is>
           <t>T2</t>
         </is>
       </c>
-      <c r="G23" s="28" t="inlineStr">
+      <c r="G26" s="31" t="inlineStr">
         <is>
           <t>Quick wins, low-hanging fruit — Past clients, sphere, sign calls</t>
         </is>
       </c>
     </row>
-    <row r="24" ht="14" customHeight="1">
-      <c r="A24" s="30" t="inlineStr"/>
-      <c r="C24" s="31" t="inlineStr">
+    <row r="27" ht="14" customHeight="1">
+      <c r="A27" s="33" t="inlineStr"/>
+      <c r="C27" s="34" t="inlineStr">
         <is>
           <t>T3</t>
         </is>
       </c>
-      <c r="D24" s="28" t="inlineStr">
+      <c r="D27" s="31" t="inlineStr">
         <is>
           <t>Volume calls, keep pipeline full — Cold calls, expired/FSBO, circle prospecting</t>
         </is>
       </c>
     </row>
-    <row r="25" ht="2" customHeight="1">
-      <c r="A25" s="1" t="n"/>
-      <c r="B25" s="1" t="n"/>
-      <c r="C25" s="1" t="n"/>
-      <c r="D25" s="1" t="n"/>
-      <c r="E25" s="1" t="n"/>
-      <c r="F25" s="1" t="n"/>
-      <c r="G25" s="1" t="n"/>
-    </row>
-    <row r="26" ht="14" customHeight="1">
-      <c r="A26" s="32" t="inlineStr">
+    <row r="28" ht="2" customHeight="1">
+      <c r="A28" s="1" t="n"/>
+      <c r="B28" s="1" t="n"/>
+      <c r="C28" s="1" t="n"/>
+      <c r="D28" s="1" t="n"/>
+      <c r="E28" s="1" t="n"/>
+      <c r="F28" s="1" t="n"/>
+      <c r="G28" s="1" t="n"/>
+    </row>
+    <row r="29" ht="14" customHeight="1">
+      <c r="A29" s="35" t="inlineStr">
         <is>
           <t xml:space="preserve">  FOLLOW-UPS</t>
         </is>
       </c>
-      <c r="D26" s="32" t="inlineStr">
+      <c r="D29" s="35" t="inlineStr">
         <is>
           <t xml:space="preserve">  APPOINTMENTS SET  #___   |   OPPORTUNITIES CREATED  #___</t>
         </is>
       </c>
     </row>
-    <row r="27" ht="12" customHeight="1">
-      <c r="A27" s="13" t="inlineStr">
+    <row r="30" ht="12" customHeight="1">
+      <c r="A30" s="15" t="inlineStr">
         <is>
           <t>NAME</t>
         </is>
       </c>
-      <c r="C27" s="13" t="inlineStr">
+      <c r="C30" s="15" t="inlineStr">
         <is>
           <t>WHY / NOTES</t>
         </is>
       </c>
-      <c r="D27" s="13" t="inlineStr">
+      <c r="D30" s="15" t="inlineStr">
         <is>
           <t>NAME / OPP.</t>
         </is>
       </c>
-      <c r="F27" s="13" t="inlineStr">
+      <c r="F30" s="15" t="inlineStr">
         <is>
           <t>NOTES</t>
         </is>
       </c>
     </row>
-    <row r="28" ht="16" customHeight="1">
-      <c r="A28" s="33" t="n"/>
-      <c r="B28" s="34" t="n"/>
-      <c r="C28" s="33" t="n"/>
-      <c r="D28" s="33" t="n"/>
-      <c r="E28" s="34" t="n"/>
-      <c r="F28" s="33" t="n"/>
-      <c r="G28" s="34" t="n"/>
-    </row>
-    <row r="29" ht="16" customHeight="1">
-      <c r="A29" s="35" t="n"/>
-      <c r="B29" s="34" t="n"/>
-      <c r="C29" s="35" t="n"/>
-      <c r="D29" s="35" t="n"/>
-      <c r="E29" s="34" t="n"/>
-      <c r="F29" s="35" t="n"/>
-      <c r="G29" s="34" t="n"/>
-    </row>
-    <row r="30" ht="16" customHeight="1">
-      <c r="A30" s="33" t="n"/>
-      <c r="B30" s="34" t="n"/>
-      <c r="C30" s="33" t="n"/>
-      <c r="D30" s="33" t="n"/>
-      <c r="E30" s="34" t="n"/>
-      <c r="F30" s="33" t="n"/>
-      <c r="G30" s="34" t="n"/>
-    </row>
     <row r="31" ht="16" customHeight="1">
-      <c r="A31" s="35" t="n"/>
-      <c r="B31" s="34" t="n"/>
-      <c r="C31" s="35" t="n"/>
-      <c r="D31" s="35" t="n"/>
-      <c r="E31" s="34" t="n"/>
-      <c r="F31" s="35" t="n"/>
-      <c r="G31" s="34" t="n"/>
+      <c r="A31" s="36" t="n"/>
+      <c r="B31" s="37" t="n"/>
+      <c r="C31" s="36" t="n"/>
+      <c r="D31" s="36" t="n"/>
+      <c r="E31" s="37" t="n"/>
+      <c r="F31" s="36" t="n"/>
+      <c r="G31" s="37" t="n"/>
     </row>
     <row r="32" ht="16" customHeight="1">
-      <c r="A32" s="33" t="n"/>
-      <c r="B32" s="34" t="n"/>
-      <c r="C32" s="33" t="n"/>
-      <c r="D32" s="33" t="n"/>
-      <c r="E32" s="34" t="n"/>
-      <c r="F32" s="33" t="n"/>
-      <c r="G32" s="34" t="n"/>
-    </row>
-    <row r="33" ht="2" customHeight="1">
-      <c r="A33" s="1" t="n"/>
-      <c r="B33" s="1" t="n"/>
-      <c r="C33" s="1" t="n"/>
-      <c r="D33" s="1" t="n"/>
-      <c r="E33" s="1" t="n"/>
-      <c r="F33" s="1" t="n"/>
-      <c r="G33" s="1" t="n"/>
+      <c r="A32" s="38" t="n"/>
+      <c r="B32" s="37" t="n"/>
+      <c r="C32" s="38" t="n"/>
+      <c r="D32" s="38" t="n"/>
+      <c r="E32" s="37" t="n"/>
+      <c r="F32" s="38" t="n"/>
+      <c r="G32" s="37" t="n"/>
+    </row>
+    <row r="33" ht="16" customHeight="1">
+      <c r="A33" s="36" t="n"/>
+      <c r="B33" s="37" t="n"/>
+      <c r="C33" s="36" t="n"/>
+      <c r="D33" s="36" t="n"/>
+      <c r="E33" s="37" t="n"/>
+      <c r="F33" s="36" t="n"/>
+      <c r="G33" s="37" t="n"/>
     </row>
     <row r="34" ht="16" customHeight="1">
-      <c r="A34" s="11" t="inlineStr">
+      <c r="A34" s="38" t="n"/>
+      <c r="B34" s="37" t="n"/>
+      <c r="C34" s="38" t="n"/>
+      <c r="D34" s="38" t="n"/>
+      <c r="E34" s="37" t="n"/>
+      <c r="F34" s="38" t="n"/>
+      <c r="G34" s="37" t="n"/>
+    </row>
+    <row r="35" ht="16" customHeight="1">
+      <c r="A35" s="36" t="n"/>
+      <c r="B35" s="37" t="n"/>
+      <c r="C35" s="36" t="n"/>
+      <c r="D35" s="36" t="n"/>
+      <c r="E35" s="37" t="n"/>
+      <c r="F35" s="36" t="n"/>
+      <c r="G35" s="37" t="n"/>
+    </row>
+    <row r="36" ht="2" customHeight="1">
+      <c r="A36" s="1" t="n"/>
+      <c r="B36" s="1" t="n"/>
+      <c r="C36" s="1" t="n"/>
+      <c r="D36" s="1" t="n"/>
+      <c r="E36" s="1" t="n"/>
+      <c r="F36" s="1" t="n"/>
+      <c r="G36" s="1" t="n"/>
+    </row>
+    <row r="37" ht="16" customHeight="1">
+      <c r="A37" s="11" t="inlineStr">
         <is>
           <t xml:space="preserve">  DAILY REVIEW</t>
         </is>
       </c>
     </row>
-    <row r="35" ht="12" customHeight="1">
-      <c r="A35" s="36" t="inlineStr">
+    <row r="38" ht="12" customHeight="1">
+      <c r="A38" s="39" t="inlineStr">
         <is>
           <t xml:space="preserve">  WHAT DIDN'T WORK?</t>
         </is>
       </c>
     </row>
-    <row r="36" ht="16" customHeight="1">
-      <c r="A36" s="37" t="inlineStr"/>
-      <c r="B36" s="38" t="n"/>
-      <c r="C36" s="38" t="n"/>
-      <c r="D36" s="38" t="n"/>
-      <c r="E36" s="38" t="n"/>
-      <c r="F36" s="38" t="n"/>
-      <c r="G36" s="38" t="n"/>
-    </row>
-    <row r="37" ht="16" customHeight="1">
-      <c r="A37" s="37" t="inlineStr"/>
-      <c r="B37" s="38" t="n"/>
-      <c r="C37" s="38" t="n"/>
-      <c r="D37" s="38" t="n"/>
-      <c r="E37" s="38" t="n"/>
-      <c r="F37" s="38" t="n"/>
-      <c r="G37" s="38" t="n"/>
-    </row>
-    <row r="38" ht="12" customHeight="1">
-      <c r="A38" s="36" t="inlineStr">
+    <row r="39" ht="16" customHeight="1">
+      <c r="A39" s="40" t="inlineStr"/>
+      <c r="B39" s="41" t="n"/>
+      <c r="C39" s="41" t="n"/>
+      <c r="D39" s="41" t="n"/>
+      <c r="E39" s="41" t="n"/>
+      <c r="F39" s="41" t="n"/>
+      <c r="G39" s="41" t="n"/>
+    </row>
+    <row r="40" ht="16" customHeight="1">
+      <c r="A40" s="40" t="inlineStr"/>
+      <c r="B40" s="41" t="n"/>
+      <c r="C40" s="41" t="n"/>
+      <c r="D40" s="41" t="n"/>
+      <c r="E40" s="41" t="n"/>
+      <c r="F40" s="41" t="n"/>
+      <c r="G40" s="41" t="n"/>
+    </row>
+    <row r="41" ht="12" customHeight="1">
+      <c r="A41" s="39" t="inlineStr">
         <is>
           <t xml:space="preserve">  WHAT WORKED TODAY?</t>
         </is>
       </c>
     </row>
-    <row r="39" ht="16" customHeight="1">
-      <c r="A39" s="37" t="inlineStr"/>
-      <c r="B39" s="38" t="n"/>
-      <c r="C39" s="38" t="n"/>
-      <c r="D39" s="38" t="n"/>
-      <c r="E39" s="38" t="n"/>
-      <c r="F39" s="38" t="n"/>
-      <c r="G39" s="38" t="n"/>
-    </row>
-    <row r="40" ht="16" customHeight="1">
-      <c r="A40" s="37" t="inlineStr"/>
-      <c r="B40" s="38" t="n"/>
-      <c r="C40" s="38" t="n"/>
-      <c r="D40" s="38" t="n"/>
-      <c r="E40" s="38" t="n"/>
-      <c r="F40" s="38" t="n"/>
-      <c r="G40" s="38" t="n"/>
-    </row>
-    <row r="41" ht="12" customHeight="1">
-      <c r="A41" s="36" t="inlineStr">
+    <row r="42" ht="16" customHeight="1">
+      <c r="A42" s="40" t="inlineStr"/>
+      <c r="B42" s="41" t="n"/>
+      <c r="C42" s="41" t="n"/>
+      <c r="D42" s="41" t="n"/>
+      <c r="E42" s="41" t="n"/>
+      <c r="F42" s="41" t="n"/>
+      <c r="G42" s="41" t="n"/>
+    </row>
+    <row r="43" ht="16" customHeight="1">
+      <c r="A43" s="40" t="inlineStr"/>
+      <c r="B43" s="41" t="n"/>
+      <c r="C43" s="41" t="n"/>
+      <c r="D43" s="41" t="n"/>
+      <c r="E43" s="41" t="n"/>
+      <c r="F43" s="41" t="n"/>
+      <c r="G43" s="41" t="n"/>
+    </row>
+    <row r="44" ht="12" customHeight="1">
+      <c r="A44" s="39" t="inlineStr">
         <is>
           <t xml:space="preserve">  WHAT WILL I IMPROVE TOMORROW?</t>
         </is>
       </c>
     </row>
-    <row r="42" ht="16" customHeight="1">
-      <c r="A42" s="37" t="inlineStr"/>
-      <c r="B42" s="38" t="n"/>
-      <c r="C42" s="38" t="n"/>
-      <c r="D42" s="38" t="n"/>
-      <c r="E42" s="38" t="n"/>
-      <c r="F42" s="38" t="n"/>
-      <c r="G42" s="38" t="n"/>
-    </row>
-    <row r="43" ht="16" customHeight="1">
-      <c r="A43" s="37" t="inlineStr"/>
-      <c r="B43" s="38" t="n"/>
-      <c r="C43" s="38" t="n"/>
-      <c r="D43" s="38" t="n"/>
-      <c r="E43" s="38" t="n"/>
-      <c r="F43" s="38" t="n"/>
-      <c r="G43" s="38" t="n"/>
-    </row>
-    <row r="44" ht="2" customHeight="1">
-      <c r="A44" s="1" t="n"/>
-      <c r="B44" s="1" t="n"/>
-      <c r="C44" s="1" t="n"/>
-      <c r="D44" s="1" t="n"/>
-      <c r="E44" s="1" t="n"/>
-      <c r="F44" s="1" t="n"/>
-      <c r="G44" s="1" t="n"/>
-    </row>
-    <row r="45" ht="12" customHeight="1">
-      <c r="A45" s="39" t="inlineStr">
+    <row r="45" ht="16" customHeight="1">
+      <c r="A45" s="40" t="inlineStr"/>
+      <c r="B45" s="41" t="n"/>
+      <c r="C45" s="41" t="n"/>
+      <c r="D45" s="41" t="n"/>
+      <c r="E45" s="41" t="n"/>
+      <c r="F45" s="41" t="n"/>
+      <c r="G45" s="41" t="n"/>
+    </row>
+    <row r="46" ht="16" customHeight="1">
+      <c r="A46" s="40" t="inlineStr"/>
+      <c r="B46" s="41" t="n"/>
+      <c r="C46" s="41" t="n"/>
+      <c r="D46" s="41" t="n"/>
+      <c r="E46" s="41" t="n"/>
+      <c r="F46" s="41" t="n"/>
+      <c r="G46" s="41" t="n"/>
+    </row>
+    <row r="47" ht="2" customHeight="1">
+      <c r="A47" s="1" t="n"/>
+      <c r="B47" s="1" t="n"/>
+      <c r="C47" s="1" t="n"/>
+      <c r="D47" s="1" t="n"/>
+      <c r="E47" s="1" t="n"/>
+      <c r="F47" s="1" t="n"/>
+      <c r="G47" s="1" t="n"/>
+    </row>
+    <row r="48" ht="12" customHeight="1">
+      <c r="A48" s="42" t="inlineStr">
         <is>
           <t>Daily Production Scoreboard  |  © 2026</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="44">
-    <mergeCell ref="A24:B24"/>
+  <mergeCells count="47">
+    <mergeCell ref="A31:B31"/>
     <mergeCell ref="A30:B30"/>
-    <mergeCell ref="F29:G29"/>
-    <mergeCell ref="A22:G22"/>
-    <mergeCell ref="A35:G35"/>
+    <mergeCell ref="D34:E34"/>
+    <mergeCell ref="F34:G34"/>
     <mergeCell ref="A4:G4"/>
-    <mergeCell ref="D24:G24"/>
     <mergeCell ref="A38:G38"/>
+    <mergeCell ref="A42:G42"/>
+    <mergeCell ref="D29:G29"/>
     <mergeCell ref="A43:G43"/>
     <mergeCell ref="D31:E31"/>
-    <mergeCell ref="A26:C26"/>
+    <mergeCell ref="A10:G10"/>
     <mergeCell ref="A2:C2"/>
-    <mergeCell ref="D26:G26"/>
+    <mergeCell ref="A44:G44"/>
     <mergeCell ref="F30:G30"/>
+    <mergeCell ref="A40:G40"/>
     <mergeCell ref="D2:E2"/>
     <mergeCell ref="A5:C5"/>
-    <mergeCell ref="A40:G40"/>
+    <mergeCell ref="A9:G9"/>
+    <mergeCell ref="D35:E35"/>
     <mergeCell ref="A39:G39"/>
-    <mergeCell ref="D27:E27"/>
-    <mergeCell ref="A34:G34"/>
+    <mergeCell ref="F33:G33"/>
+    <mergeCell ref="A48:G48"/>
     <mergeCell ref="D32:E32"/>
     <mergeCell ref="F32:G32"/>
+    <mergeCell ref="A29:C29"/>
     <mergeCell ref="A27:B27"/>
+    <mergeCell ref="F35:G35"/>
     <mergeCell ref="A45:G45"/>
     <mergeCell ref="F8:G8"/>
-    <mergeCell ref="A36:G36"/>
     <mergeCell ref="F2:G2"/>
+    <mergeCell ref="A26:B26"/>
+    <mergeCell ref="A33:B33"/>
     <mergeCell ref="F31:G31"/>
-    <mergeCell ref="D28:E28"/>
     <mergeCell ref="A32:B32"/>
-    <mergeCell ref="F28:G28"/>
-    <mergeCell ref="A23:B23"/>
+    <mergeCell ref="A16:G16"/>
     <mergeCell ref="A8:E8"/>
+    <mergeCell ref="D27:G27"/>
     <mergeCell ref="A41:G41"/>
-    <mergeCell ref="F27:G27"/>
+    <mergeCell ref="A35:B35"/>
     <mergeCell ref="A37:G37"/>
-    <mergeCell ref="A29:B29"/>
+    <mergeCell ref="A46:G46"/>
     <mergeCell ref="D30:E30"/>
-    <mergeCell ref="D29:E29"/>
+    <mergeCell ref="D33:E33"/>
+    <mergeCell ref="A21:G21"/>
     <mergeCell ref="A6:C6"/>
-    <mergeCell ref="D23:E23"/>
-    <mergeCell ref="A28:B28"/>
-    <mergeCell ref="A31:B31"/>
-    <mergeCell ref="A42:G42"/>
+    <mergeCell ref="D26:E26"/>
+    <mergeCell ref="A34:B34"/>
   </mergeCells>
   <pageMargins left="0.3" right="0.3" top="0.25" bottom="0.25" header="0.05" footer="0.05"/>
   <pageSetup orientation="portrait" paperSize="1" fitToHeight="1" fitToWidth="1"/>

</xml_diff>

<commit_message>
Style T1/T2/T3 as colored badges in call log tier column (web, PDF, Excel)
</commit_message>
<xml_diff>
--- a/Daily_Production_Scoreboard_v6.xlsx
+++ b/Daily_Production_Scoreboard_v6.xlsx
@@ -19,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="20">
+  <fonts count="19">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -102,11 +102,6 @@
       <name val="Calibri"/>
       <color rgb="00CCCCCC"/>
       <sz val="7"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <color rgb="00CCCCCC"/>
-      <sz val="6.5"/>
     </font>
     <font>
       <name val="Calibri"/>
@@ -246,7 +241,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="43">
+  <cellXfs count="42">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -301,9 +296,6 @@
     <xf numFmtId="0" fontId="14" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="13" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -311,35 +303,35 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="14" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="12" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="15" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="9" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="16" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="9" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="9" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="9" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="16" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="12" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -351,11 +343,11 @@
     <xf numFmtId="0" fontId="8" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="3" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="18" fillId="3" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="15" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="14" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -888,79 +880,227 @@
         <v>1</v>
       </c>
       <c r="B12" s="18" t="n"/>
-      <c r="C12" s="19" t="inlineStr">
-        <is>
-          <t>T1  T2  T3</t>
-        </is>
-      </c>
-      <c r="D12" s="20" t="inlineStr">
+      <c r="C12" s="9" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <b val="1"/>
+              <color rgb="00555555"/>
+              <sz val="65"/>
+            </rPr>
+            <t>T1</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="00CCCCCC"/>
+              <sz val="65"/>
+            </rPr>
+            <t>  </t>
+          </r>
+          <r>
+            <rPr>
+              <b val="1"/>
+              <color rgb="00999999"/>
+              <sz val="65"/>
+            </rPr>
+            <t>T2</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="00CCCCCC"/>
+              <sz val="65"/>
+            </rPr>
+            <t>  </t>
+          </r>
+          <r>
+            <rPr>
+              <b val="1"/>
+              <color rgb="00BBBBBB"/>
+              <sz val="65"/>
+            </rPr>
+            <t>T3</t>
+          </r>
+        </is>
+      </c>
+      <c r="D12" s="19" t="inlineStr">
         <is>
           <t>S  VM  A  NA  B  CB</t>
         </is>
       </c>
       <c r="E12" s="18" t="n"/>
-      <c r="F12" s="21" t="n"/>
-      <c r="G12" s="21" t="n"/>
+      <c r="F12" s="20" t="n"/>
+      <c r="G12" s="20" t="n"/>
     </row>
     <row r="13" ht="18" customHeight="1">
-      <c r="A13" s="22" t="n">
+      <c r="A13" s="21" t="n">
         <v>2</v>
       </c>
-      <c r="B13" s="23" t="n"/>
-      <c r="C13" s="24" t="inlineStr">
-        <is>
-          <t>T1  T2  T3</t>
-        </is>
-      </c>
-      <c r="D13" s="25" t="inlineStr">
+      <c r="B13" s="22" t="n"/>
+      <c r="C13" s="23" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <b val="1"/>
+              <color rgb="00555555"/>
+              <sz val="65"/>
+            </rPr>
+            <t>T1</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="00CCCCCC"/>
+              <sz val="65"/>
+            </rPr>
+            <t>  </t>
+          </r>
+          <r>
+            <rPr>
+              <b val="1"/>
+              <color rgb="00999999"/>
+              <sz val="65"/>
+            </rPr>
+            <t>T2</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="00CCCCCC"/>
+              <sz val="65"/>
+            </rPr>
+            <t>  </t>
+          </r>
+          <r>
+            <rPr>
+              <b val="1"/>
+              <color rgb="00BBBBBB"/>
+              <sz val="65"/>
+            </rPr>
+            <t>T3</t>
+          </r>
+        </is>
+      </c>
+      <c r="D13" s="24" t="inlineStr">
         <is>
           <t>S  VM  A  NA  B  CB</t>
         </is>
       </c>
-      <c r="E13" s="23" t="n"/>
-      <c r="F13" s="26" t="n"/>
-      <c r="G13" s="26" t="n"/>
+      <c r="E13" s="22" t="n"/>
+      <c r="F13" s="25" t="n"/>
+      <c r="G13" s="25" t="n"/>
     </row>
     <row r="14" ht="18" customHeight="1">
       <c r="A14" s="17" t="n">
         <v>3</v>
       </c>
       <c r="B14" s="18" t="n"/>
-      <c r="C14" s="19" t="inlineStr">
-        <is>
-          <t>T1  T2  T3</t>
-        </is>
-      </c>
-      <c r="D14" s="20" t="inlineStr">
+      <c r="C14" s="9" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <b val="1"/>
+              <color rgb="00555555"/>
+              <sz val="65"/>
+            </rPr>
+            <t>T1</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="00CCCCCC"/>
+              <sz val="65"/>
+            </rPr>
+            <t>  </t>
+          </r>
+          <r>
+            <rPr>
+              <b val="1"/>
+              <color rgb="00999999"/>
+              <sz val="65"/>
+            </rPr>
+            <t>T2</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="00CCCCCC"/>
+              <sz val="65"/>
+            </rPr>
+            <t>  </t>
+          </r>
+          <r>
+            <rPr>
+              <b val="1"/>
+              <color rgb="00BBBBBB"/>
+              <sz val="65"/>
+            </rPr>
+            <t>T3</t>
+          </r>
+        </is>
+      </c>
+      <c r="D14" s="19" t="inlineStr">
         <is>
           <t>S  VM  A  NA  B  CB</t>
         </is>
       </c>
       <c r="E14" s="18" t="n"/>
-      <c r="F14" s="21" t="n"/>
-      <c r="G14" s="21" t="n"/>
+      <c r="F14" s="20" t="n"/>
+      <c r="G14" s="20" t="n"/>
     </row>
     <row r="15" ht="18" customHeight="1">
-      <c r="A15" s="22" t="n">
+      <c r="A15" s="21" t="n">
         <v>4</v>
       </c>
-      <c r="B15" s="23" t="n"/>
-      <c r="C15" s="24" t="inlineStr">
-        <is>
-          <t>T1  T2  T3</t>
-        </is>
-      </c>
-      <c r="D15" s="25" t="inlineStr">
+      <c r="B15" s="22" t="n"/>
+      <c r="C15" s="23" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <b val="1"/>
+              <color rgb="00555555"/>
+              <sz val="65"/>
+            </rPr>
+            <t>T1</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="00CCCCCC"/>
+              <sz val="65"/>
+            </rPr>
+            <t>  </t>
+          </r>
+          <r>
+            <rPr>
+              <b val="1"/>
+              <color rgb="00999999"/>
+              <sz val="65"/>
+            </rPr>
+            <t>T2</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="00CCCCCC"/>
+              <sz val="65"/>
+            </rPr>
+            <t>  </t>
+          </r>
+          <r>
+            <rPr>
+              <b val="1"/>
+              <color rgb="00BBBBBB"/>
+              <sz val="65"/>
+            </rPr>
+            <t>T3</t>
+          </r>
+        </is>
+      </c>
+      <c r="D15" s="24" t="inlineStr">
         <is>
           <t>S  VM  A  NA  B  CB</t>
         </is>
       </c>
-      <c r="E15" s="23" t="n"/>
-      <c r="F15" s="26" t="n"/>
-      <c r="G15" s="26" t="n"/>
+      <c r="E15" s="22" t="n"/>
+      <c r="F15" s="25" t="n"/>
+      <c r="G15" s="25" t="n"/>
     </row>
     <row r="16" ht="11" customHeight="1">
-      <c r="A16" s="27" t="inlineStr">
+      <c r="A16" s="26" t="inlineStr">
         <is>
           <t xml:space="preserve">  Tier 2 (Second 30 min) — Quick wins: past clients, sphere, sign calls</t>
         </is>
@@ -971,79 +1111,227 @@
         <v>5</v>
       </c>
       <c r="B17" s="18" t="n"/>
-      <c r="C17" s="19" t="inlineStr">
-        <is>
-          <t>T1  T2  T3</t>
-        </is>
-      </c>
-      <c r="D17" s="20" t="inlineStr">
+      <c r="C17" s="9" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <b val="1"/>
+              <color rgb="00555555"/>
+              <sz val="65"/>
+            </rPr>
+            <t>T1</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="00CCCCCC"/>
+              <sz val="65"/>
+            </rPr>
+            <t>  </t>
+          </r>
+          <r>
+            <rPr>
+              <b val="1"/>
+              <color rgb="00999999"/>
+              <sz val="65"/>
+            </rPr>
+            <t>T2</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="00CCCCCC"/>
+              <sz val="65"/>
+            </rPr>
+            <t>  </t>
+          </r>
+          <r>
+            <rPr>
+              <b val="1"/>
+              <color rgb="00BBBBBB"/>
+              <sz val="65"/>
+            </rPr>
+            <t>T3</t>
+          </r>
+        </is>
+      </c>
+      <c r="D17" s="19" t="inlineStr">
         <is>
           <t>S  VM  A  NA  B  CB</t>
         </is>
       </c>
       <c r="E17" s="18" t="n"/>
-      <c r="F17" s="21" t="n"/>
-      <c r="G17" s="21" t="n"/>
+      <c r="F17" s="20" t="n"/>
+      <c r="G17" s="20" t="n"/>
     </row>
     <row r="18" ht="18" customHeight="1">
-      <c r="A18" s="22" t="n">
+      <c r="A18" s="21" t="n">
         <v>6</v>
       </c>
-      <c r="B18" s="23" t="n"/>
-      <c r="C18" s="24" t="inlineStr">
-        <is>
-          <t>T1  T2  T3</t>
-        </is>
-      </c>
-      <c r="D18" s="25" t="inlineStr">
+      <c r="B18" s="22" t="n"/>
+      <c r="C18" s="23" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <b val="1"/>
+              <color rgb="00555555"/>
+              <sz val="65"/>
+            </rPr>
+            <t>T1</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="00CCCCCC"/>
+              <sz val="65"/>
+            </rPr>
+            <t>  </t>
+          </r>
+          <r>
+            <rPr>
+              <b val="1"/>
+              <color rgb="00999999"/>
+              <sz val="65"/>
+            </rPr>
+            <t>T2</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="00CCCCCC"/>
+              <sz val="65"/>
+            </rPr>
+            <t>  </t>
+          </r>
+          <r>
+            <rPr>
+              <b val="1"/>
+              <color rgb="00BBBBBB"/>
+              <sz val="65"/>
+            </rPr>
+            <t>T3</t>
+          </r>
+        </is>
+      </c>
+      <c r="D18" s="24" t="inlineStr">
         <is>
           <t>S  VM  A  NA  B  CB</t>
         </is>
       </c>
-      <c r="E18" s="23" t="n"/>
-      <c r="F18" s="26" t="n"/>
-      <c r="G18" s="26" t="n"/>
+      <c r="E18" s="22" t="n"/>
+      <c r="F18" s="25" t="n"/>
+      <c r="G18" s="25" t="n"/>
     </row>
     <row r="19" ht="18" customHeight="1">
       <c r="A19" s="17" t="n">
         <v>7</v>
       </c>
       <c r="B19" s="18" t="n"/>
-      <c r="C19" s="19" t="inlineStr">
-        <is>
-          <t>T1  T2  T3</t>
-        </is>
-      </c>
-      <c r="D19" s="20" t="inlineStr">
+      <c r="C19" s="9" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <b val="1"/>
+              <color rgb="00555555"/>
+              <sz val="65"/>
+            </rPr>
+            <t>T1</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="00CCCCCC"/>
+              <sz val="65"/>
+            </rPr>
+            <t>  </t>
+          </r>
+          <r>
+            <rPr>
+              <b val="1"/>
+              <color rgb="00999999"/>
+              <sz val="65"/>
+            </rPr>
+            <t>T2</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="00CCCCCC"/>
+              <sz val="65"/>
+            </rPr>
+            <t>  </t>
+          </r>
+          <r>
+            <rPr>
+              <b val="1"/>
+              <color rgb="00BBBBBB"/>
+              <sz val="65"/>
+            </rPr>
+            <t>T3</t>
+          </r>
+        </is>
+      </c>
+      <c r="D19" s="19" t="inlineStr">
         <is>
           <t>S  VM  A  NA  B  CB</t>
         </is>
       </c>
       <c r="E19" s="18" t="n"/>
-      <c r="F19" s="21" t="n"/>
-      <c r="G19" s="21" t="n"/>
+      <c r="F19" s="20" t="n"/>
+      <c r="G19" s="20" t="n"/>
     </row>
     <row r="20" ht="18" customHeight="1">
-      <c r="A20" s="22" t="n">
+      <c r="A20" s="21" t="n">
         <v>8</v>
       </c>
-      <c r="B20" s="23" t="n"/>
-      <c r="C20" s="24" t="inlineStr">
-        <is>
-          <t>T1  T2  T3</t>
-        </is>
-      </c>
-      <c r="D20" s="25" t="inlineStr">
+      <c r="B20" s="22" t="n"/>
+      <c r="C20" s="23" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <b val="1"/>
+              <color rgb="00555555"/>
+              <sz val="65"/>
+            </rPr>
+            <t>T1</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="00CCCCCC"/>
+              <sz val="65"/>
+            </rPr>
+            <t>  </t>
+          </r>
+          <r>
+            <rPr>
+              <b val="1"/>
+              <color rgb="00999999"/>
+              <sz val="65"/>
+            </rPr>
+            <t>T2</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="00CCCCCC"/>
+              <sz val="65"/>
+            </rPr>
+            <t>  </t>
+          </r>
+          <r>
+            <rPr>
+              <b val="1"/>
+              <color rgb="00BBBBBB"/>
+              <sz val="65"/>
+            </rPr>
+            <t>T3</t>
+          </r>
+        </is>
+      </c>
+      <c r="D20" s="24" t="inlineStr">
         <is>
           <t>S  VM  A  NA  B  CB</t>
         </is>
       </c>
-      <c r="E20" s="23" t="n"/>
-      <c r="F20" s="26" t="n"/>
-      <c r="G20" s="26" t="n"/>
+      <c r="E20" s="22" t="n"/>
+      <c r="F20" s="25" t="n"/>
+      <c r="G20" s="25" t="n"/>
     </row>
     <row r="21" ht="14" customHeight="1">
-      <c r="A21" s="28" t="inlineStr">
+      <c r="A21" s="27" t="inlineStr">
         <is>
           <t>⏰  BLOCK 2 — The Cleanup: 4:30 – 5:00 PM  •  Circling back on earlier calls &amp; callbacks</t>
         </is>
@@ -1054,112 +1342,260 @@
         <v>9</v>
       </c>
       <c r="B22" s="18" t="n"/>
-      <c r="C22" s="19" t="inlineStr">
-        <is>
-          <t>T1  T2  T3</t>
-        </is>
-      </c>
-      <c r="D22" s="20" t="inlineStr">
+      <c r="C22" s="9" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <b val="1"/>
+              <color rgb="00555555"/>
+              <sz val="65"/>
+            </rPr>
+            <t>T1</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="00CCCCCC"/>
+              <sz val="65"/>
+            </rPr>
+            <t>  </t>
+          </r>
+          <r>
+            <rPr>
+              <b val="1"/>
+              <color rgb="00999999"/>
+              <sz val="65"/>
+            </rPr>
+            <t>T2</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="00CCCCCC"/>
+              <sz val="65"/>
+            </rPr>
+            <t>  </t>
+          </r>
+          <r>
+            <rPr>
+              <b val="1"/>
+              <color rgb="00BBBBBB"/>
+              <sz val="65"/>
+            </rPr>
+            <t>T3</t>
+          </r>
+        </is>
+      </c>
+      <c r="D22" s="19" t="inlineStr">
         <is>
           <t>S  VM  A  NA  B  CB</t>
         </is>
       </c>
       <c r="E22" s="18" t="n"/>
-      <c r="F22" s="21" t="n"/>
-      <c r="G22" s="21" t="n"/>
+      <c r="F22" s="20" t="n"/>
+      <c r="G22" s="20" t="n"/>
     </row>
     <row r="23" ht="18" customHeight="1">
-      <c r="A23" s="22" t="n">
+      <c r="A23" s="21" t="n">
         <v>10</v>
       </c>
-      <c r="B23" s="23" t="n"/>
-      <c r="C23" s="24" t="inlineStr">
-        <is>
-          <t>T1  T2  T3</t>
-        </is>
-      </c>
-      <c r="D23" s="25" t="inlineStr">
+      <c r="B23" s="22" t="n"/>
+      <c r="C23" s="23" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <b val="1"/>
+              <color rgb="00555555"/>
+              <sz val="65"/>
+            </rPr>
+            <t>T1</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="00CCCCCC"/>
+              <sz val="65"/>
+            </rPr>
+            <t>  </t>
+          </r>
+          <r>
+            <rPr>
+              <b val="1"/>
+              <color rgb="00999999"/>
+              <sz val="65"/>
+            </rPr>
+            <t>T2</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="00CCCCCC"/>
+              <sz val="65"/>
+            </rPr>
+            <t>  </t>
+          </r>
+          <r>
+            <rPr>
+              <b val="1"/>
+              <color rgb="00BBBBBB"/>
+              <sz val="65"/>
+            </rPr>
+            <t>T3</t>
+          </r>
+        </is>
+      </c>
+      <c r="D23" s="24" t="inlineStr">
         <is>
           <t>S  VM  A  NA  B  CB</t>
         </is>
       </c>
-      <c r="E23" s="23" t="n"/>
-      <c r="F23" s="26" t="n"/>
-      <c r="G23" s="26" t="n"/>
+      <c r="E23" s="22" t="n"/>
+      <c r="F23" s="25" t="n"/>
+      <c r="G23" s="25" t="n"/>
     </row>
     <row r="24" ht="18" customHeight="1">
       <c r="A24" s="17" t="n">
         <v>11</v>
       </c>
       <c r="B24" s="18" t="n"/>
-      <c r="C24" s="19" t="inlineStr">
-        <is>
-          <t>T1  T2  T3</t>
-        </is>
-      </c>
-      <c r="D24" s="20" t="inlineStr">
+      <c r="C24" s="9" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <b val="1"/>
+              <color rgb="00555555"/>
+              <sz val="65"/>
+            </rPr>
+            <t>T1</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="00CCCCCC"/>
+              <sz val="65"/>
+            </rPr>
+            <t>  </t>
+          </r>
+          <r>
+            <rPr>
+              <b val="1"/>
+              <color rgb="00999999"/>
+              <sz val="65"/>
+            </rPr>
+            <t>T2</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="00CCCCCC"/>
+              <sz val="65"/>
+            </rPr>
+            <t>  </t>
+          </r>
+          <r>
+            <rPr>
+              <b val="1"/>
+              <color rgb="00BBBBBB"/>
+              <sz val="65"/>
+            </rPr>
+            <t>T3</t>
+          </r>
+        </is>
+      </c>
+      <c r="D24" s="19" t="inlineStr">
         <is>
           <t>S  VM  A  NA  B  CB</t>
         </is>
       </c>
       <c r="E24" s="18" t="n"/>
-      <c r="F24" s="21" t="n"/>
-      <c r="G24" s="21" t="n"/>
+      <c r="F24" s="20" t="n"/>
+      <c r="G24" s="20" t="n"/>
     </row>
     <row r="25" ht="18" customHeight="1">
-      <c r="A25" s="22" t="n">
+      <c r="A25" s="21" t="n">
         <v>12</v>
       </c>
-      <c r="B25" s="23" t="n"/>
-      <c r="C25" s="24" t="inlineStr">
-        <is>
-          <t>T1  T2  T3</t>
-        </is>
-      </c>
-      <c r="D25" s="25" t="inlineStr">
+      <c r="B25" s="22" t="n"/>
+      <c r="C25" s="23" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <b val="1"/>
+              <color rgb="00555555"/>
+              <sz val="65"/>
+            </rPr>
+            <t>T1</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="00CCCCCC"/>
+              <sz val="65"/>
+            </rPr>
+            <t>  </t>
+          </r>
+          <r>
+            <rPr>
+              <b val="1"/>
+              <color rgb="00999999"/>
+              <sz val="65"/>
+            </rPr>
+            <t>T2</t>
+          </r>
+          <r>
+            <rPr>
+              <color rgb="00CCCCCC"/>
+              <sz val="65"/>
+            </rPr>
+            <t>  </t>
+          </r>
+          <r>
+            <rPr>
+              <b val="1"/>
+              <color rgb="00BBBBBB"/>
+              <sz val="65"/>
+            </rPr>
+            <t>T3</t>
+          </r>
+        </is>
+      </c>
+      <c r="D25" s="24" t="inlineStr">
         <is>
           <t>S  VM  A  NA  B  CB</t>
         </is>
       </c>
-      <c r="E25" s="23" t="n"/>
-      <c r="F25" s="26" t="n"/>
-      <c r="G25" s="26" t="n"/>
+      <c r="E25" s="22" t="n"/>
+      <c r="F25" s="25" t="n"/>
+      <c r="G25" s="25" t="n"/>
     </row>
     <row r="26" ht="22" customHeight="1">
-      <c r="A26" s="29" t="inlineStr">
+      <c r="A26" s="28" t="inlineStr">
         <is>
           <t>TIER REFERENCE</t>
         </is>
       </c>
-      <c r="C26" s="30" t="inlineStr">
+      <c r="C26" s="29" t="inlineStr">
         <is>
           <t>T1</t>
         </is>
       </c>
-      <c r="D26" s="31" t="inlineStr">
+      <c r="D26" s="30" t="inlineStr">
         <is>
           <t>Convert fast - highest priority — Active buyers/sellers, referrals, warm follow-ups</t>
         </is>
       </c>
-      <c r="F26" s="32" t="inlineStr">
+      <c r="F26" s="31" t="inlineStr">
         <is>
           <t>T2</t>
         </is>
       </c>
-      <c r="G26" s="31" t="inlineStr">
+      <c r="G26" s="30" t="inlineStr">
         <is>
           <t>Quick wins, low-hanging fruit — Past clients, sphere, sign calls</t>
         </is>
       </c>
     </row>
     <row r="27" ht="14" customHeight="1">
-      <c r="A27" s="33" t="inlineStr"/>
-      <c r="C27" s="34" t="inlineStr">
+      <c r="A27" s="32" t="inlineStr"/>
+      <c r="C27" s="33" t="inlineStr">
         <is>
           <t>T3</t>
         </is>
       </c>
-      <c r="D27" s="31" t="inlineStr">
+      <c r="D27" s="30" t="inlineStr">
         <is>
           <t>Volume calls, keep pipeline full — Cold calls, expired/FSBO, circle prospecting</t>
         </is>
@@ -1175,12 +1611,12 @@
       <c r="G28" s="1" t="n"/>
     </row>
     <row r="29" ht="14" customHeight="1">
-      <c r="A29" s="35" t="inlineStr">
+      <c r="A29" s="34" t="inlineStr">
         <is>
           <t xml:space="preserve">  FOLLOW-UPS</t>
         </is>
       </c>
-      <c r="D29" s="35" t="inlineStr">
+      <c r="D29" s="34" t="inlineStr">
         <is>
           <t xml:space="preserve">  APPOINTMENTS SET  #___   |   OPPORTUNITIES CREATED  #___</t>
         </is>
@@ -1209,49 +1645,49 @@
       </c>
     </row>
     <row r="31" ht="16" customHeight="1">
-      <c r="A31" s="36" t="n"/>
-      <c r="B31" s="37" t="n"/>
-      <c r="C31" s="36" t="n"/>
-      <c r="D31" s="36" t="n"/>
-      <c r="E31" s="37" t="n"/>
-      <c r="F31" s="36" t="n"/>
-      <c r="G31" s="37" t="n"/>
+      <c r="A31" s="35" t="n"/>
+      <c r="B31" s="36" t="n"/>
+      <c r="C31" s="35" t="n"/>
+      <c r="D31" s="35" t="n"/>
+      <c r="E31" s="36" t="n"/>
+      <c r="F31" s="35" t="n"/>
+      <c r="G31" s="36" t="n"/>
     </row>
     <row r="32" ht="16" customHeight="1">
-      <c r="A32" s="38" t="n"/>
-      <c r="B32" s="37" t="n"/>
-      <c r="C32" s="38" t="n"/>
-      <c r="D32" s="38" t="n"/>
-      <c r="E32" s="37" t="n"/>
-      <c r="F32" s="38" t="n"/>
-      <c r="G32" s="37" t="n"/>
+      <c r="A32" s="37" t="n"/>
+      <c r="B32" s="36" t="n"/>
+      <c r="C32" s="37" t="n"/>
+      <c r="D32" s="37" t="n"/>
+      <c r="E32" s="36" t="n"/>
+      <c r="F32" s="37" t="n"/>
+      <c r="G32" s="36" t="n"/>
     </row>
     <row r="33" ht="16" customHeight="1">
-      <c r="A33" s="36" t="n"/>
-      <c r="B33" s="37" t="n"/>
-      <c r="C33" s="36" t="n"/>
-      <c r="D33" s="36" t="n"/>
-      <c r="E33" s="37" t="n"/>
-      <c r="F33" s="36" t="n"/>
-      <c r="G33" s="37" t="n"/>
+      <c r="A33" s="35" t="n"/>
+      <c r="B33" s="36" t="n"/>
+      <c r="C33" s="35" t="n"/>
+      <c r="D33" s="35" t="n"/>
+      <c r="E33" s="36" t="n"/>
+      <c r="F33" s="35" t="n"/>
+      <c r="G33" s="36" t="n"/>
     </row>
     <row r="34" ht="16" customHeight="1">
-      <c r="A34" s="38" t="n"/>
-      <c r="B34" s="37" t="n"/>
-      <c r="C34" s="38" t="n"/>
-      <c r="D34" s="38" t="n"/>
-      <c r="E34" s="37" t="n"/>
-      <c r="F34" s="38" t="n"/>
-      <c r="G34" s="37" t="n"/>
+      <c r="A34" s="37" t="n"/>
+      <c r="B34" s="36" t="n"/>
+      <c r="C34" s="37" t="n"/>
+      <c r="D34" s="37" t="n"/>
+      <c r="E34" s="36" t="n"/>
+      <c r="F34" s="37" t="n"/>
+      <c r="G34" s="36" t="n"/>
     </row>
     <row r="35" ht="16" customHeight="1">
-      <c r="A35" s="36" t="n"/>
-      <c r="B35" s="37" t="n"/>
-      <c r="C35" s="36" t="n"/>
-      <c r="D35" s="36" t="n"/>
-      <c r="E35" s="37" t="n"/>
-      <c r="F35" s="36" t="n"/>
-      <c r="G35" s="37" t="n"/>
+      <c r="A35" s="35" t="n"/>
+      <c r="B35" s="36" t="n"/>
+      <c r="C35" s="35" t="n"/>
+      <c r="D35" s="35" t="n"/>
+      <c r="E35" s="36" t="n"/>
+      <c r="F35" s="35" t="n"/>
+      <c r="G35" s="36" t="n"/>
     </row>
     <row r="36" ht="2" customHeight="1">
       <c r="A36" s="1" t="n"/>
@@ -1270,79 +1706,79 @@
       </c>
     </row>
     <row r="38" ht="12" customHeight="1">
-      <c r="A38" s="39" t="inlineStr">
+      <c r="A38" s="38" t="inlineStr">
         <is>
           <t xml:space="preserve">  WHAT DIDN'T WORK?</t>
         </is>
       </c>
     </row>
     <row r="39" ht="16" customHeight="1">
-      <c r="A39" s="40" t="inlineStr"/>
-      <c r="B39" s="41" t="n"/>
-      <c r="C39" s="41" t="n"/>
-      <c r="D39" s="41" t="n"/>
-      <c r="E39" s="41" t="n"/>
-      <c r="F39" s="41" t="n"/>
-      <c r="G39" s="41" t="n"/>
+      <c r="A39" s="39" t="inlineStr"/>
+      <c r="B39" s="40" t="n"/>
+      <c r="C39" s="40" t="n"/>
+      <c r="D39" s="40" t="n"/>
+      <c r="E39" s="40" t="n"/>
+      <c r="F39" s="40" t="n"/>
+      <c r="G39" s="40" t="n"/>
     </row>
     <row r="40" ht="16" customHeight="1">
-      <c r="A40" s="40" t="inlineStr"/>
-      <c r="B40" s="41" t="n"/>
-      <c r="C40" s="41" t="n"/>
-      <c r="D40" s="41" t="n"/>
-      <c r="E40" s="41" t="n"/>
-      <c r="F40" s="41" t="n"/>
-      <c r="G40" s="41" t="n"/>
+      <c r="A40" s="39" t="inlineStr"/>
+      <c r="B40" s="40" t="n"/>
+      <c r="C40" s="40" t="n"/>
+      <c r="D40" s="40" t="n"/>
+      <c r="E40" s="40" t="n"/>
+      <c r="F40" s="40" t="n"/>
+      <c r="G40" s="40" t="n"/>
     </row>
     <row r="41" ht="12" customHeight="1">
-      <c r="A41" s="39" t="inlineStr">
+      <c r="A41" s="38" t="inlineStr">
         <is>
           <t xml:space="preserve">  WHAT WORKED TODAY?</t>
         </is>
       </c>
     </row>
     <row r="42" ht="16" customHeight="1">
-      <c r="A42" s="40" t="inlineStr"/>
-      <c r="B42" s="41" t="n"/>
-      <c r="C42" s="41" t="n"/>
-      <c r="D42" s="41" t="n"/>
-      <c r="E42" s="41" t="n"/>
-      <c r="F42" s="41" t="n"/>
-      <c r="G42" s="41" t="n"/>
+      <c r="A42" s="39" t="inlineStr"/>
+      <c r="B42" s="40" t="n"/>
+      <c r="C42" s="40" t="n"/>
+      <c r="D42" s="40" t="n"/>
+      <c r="E42" s="40" t="n"/>
+      <c r="F42" s="40" t="n"/>
+      <c r="G42" s="40" t="n"/>
     </row>
     <row r="43" ht="16" customHeight="1">
-      <c r="A43" s="40" t="inlineStr"/>
-      <c r="B43" s="41" t="n"/>
-      <c r="C43" s="41" t="n"/>
-      <c r="D43" s="41" t="n"/>
-      <c r="E43" s="41" t="n"/>
-      <c r="F43" s="41" t="n"/>
-      <c r="G43" s="41" t="n"/>
+      <c r="A43" s="39" t="inlineStr"/>
+      <c r="B43" s="40" t="n"/>
+      <c r="C43" s="40" t="n"/>
+      <c r="D43" s="40" t="n"/>
+      <c r="E43" s="40" t="n"/>
+      <c r="F43" s="40" t="n"/>
+      <c r="G43" s="40" t="n"/>
     </row>
     <row r="44" ht="12" customHeight="1">
-      <c r="A44" s="39" t="inlineStr">
+      <c r="A44" s="38" t="inlineStr">
         <is>
           <t xml:space="preserve">  WHAT WILL I IMPROVE TOMORROW?</t>
         </is>
       </c>
     </row>
     <row r="45" ht="16" customHeight="1">
-      <c r="A45" s="40" t="inlineStr"/>
-      <c r="B45" s="41" t="n"/>
-      <c r="C45" s="41" t="n"/>
-      <c r="D45" s="41" t="n"/>
-      <c r="E45" s="41" t="n"/>
-      <c r="F45" s="41" t="n"/>
-      <c r="G45" s="41" t="n"/>
+      <c r="A45" s="39" t="inlineStr"/>
+      <c r="B45" s="40" t="n"/>
+      <c r="C45" s="40" t="n"/>
+      <c r="D45" s="40" t="n"/>
+      <c r="E45" s="40" t="n"/>
+      <c r="F45" s="40" t="n"/>
+      <c r="G45" s="40" t="n"/>
     </row>
     <row r="46" ht="16" customHeight="1">
-      <c r="A46" s="40" t="inlineStr"/>
-      <c r="B46" s="41" t="n"/>
-      <c r="C46" s="41" t="n"/>
-      <c r="D46" s="41" t="n"/>
-      <c r="E46" s="41" t="n"/>
-      <c r="F46" s="41" t="n"/>
-      <c r="G46" s="41" t="n"/>
+      <c r="A46" s="39" t="inlineStr"/>
+      <c r="B46" s="40" t="n"/>
+      <c r="C46" s="40" t="n"/>
+      <c r="D46" s="40" t="n"/>
+      <c r="E46" s="40" t="n"/>
+      <c r="F46" s="40" t="n"/>
+      <c r="G46" s="40" t="n"/>
     </row>
     <row r="47" ht="2" customHeight="1">
       <c r="A47" s="1" t="n"/>
@@ -1354,7 +1790,7 @@
       <c r="G47" s="1" t="n"/>
     </row>
     <row r="48" ht="12" customHeight="1">
-      <c r="A48" s="42" t="inlineStr">
+      <c r="A48" s="41" t="inlineStr">
         <is>
           <t>Daily Production Scoreboard  |  © 2026</t>
         </is>

</xml_diff>